<commit_message>
Metrado Varones: acero solo donde H supera 0.40 m desde el NCT; tramos tapados siempre con acero de cuerpo y tapa
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
@@ -17480,21 +17480,21 @@
       </c>
       <c r="D11" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E11" s="106" t="inlineStr">
         <is>
-          <t>SEC 01</t>
+          <t>SEC 02</t>
         </is>
       </c>
       <c r="F11" s="106" t="inlineStr">
         <is>
-          <t>SEC 02</t>
+          <t>SEC 03</t>
         </is>
       </c>
       <c r="G11" s="107" t="n">
-        <v>13.2</v>
+        <v>6</v>
       </c>
       <c r="H11" s="106" t="inlineStr">
         <is>
@@ -17509,7 +17509,7 @@
         <v>0.2</v>
       </c>
       <c r="K11" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L11" s="107" t="n">
         <v>7</v>
@@ -17530,10 +17530,10 @@
         <v>0.25</v>
       </c>
       <c r="Q11" s="107" t="n">
-        <v>1.3</v>
+        <v>1.44</v>
       </c>
       <c r="R11" s="107" t="n">
-        <v>1.44</v>
+        <v>1.5</v>
       </c>
       <c r="S11" s="141">
         <f>IF(B11="","",(Q11+R11)/2)</f>
@@ -17555,11 +17555,23 @@
         <f>IF(B11="","",O11+V11)</f>
         <v/>
       </c>
-      <c r="X11" s="142" t="n"/>
-      <c r="Y11" s="353" t="inlineStr"/>
-      <c r="Z11" s="144" t="n"/>
-      <c r="AA11" s="144" t="n"/>
-      <c r="AB11" s="144" t="n"/>
+      <c r="X11" s="142" t="inlineStr">
+        <is>
+          <t>3/8"</t>
+        </is>
+      </c>
+      <c r="Y11" s="353" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="Z11" s="144" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AA11" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB11" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="AC11" s="108">
         <f>IF(B11="","",IF(D11="TAPADA",(AA11+AB11)/2,0))</f>
         <v/>
@@ -17597,21 +17609,21 @@
       </c>
       <c r="D12" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E12" s="106" t="inlineStr">
         <is>
-          <t>SEC 02</t>
+          <t>SEC 03</t>
         </is>
       </c>
       <c r="F12" s="106" t="inlineStr">
         <is>
-          <t>SEC 03</t>
+          <t>SEC 04</t>
         </is>
       </c>
       <c r="G12" s="107" t="n">
-        <v>6</v>
+        <v>58.1</v>
       </c>
       <c r="H12" s="106" t="inlineStr">
         <is>
@@ -17623,13 +17635,13 @@
         <v/>
       </c>
       <c r="J12" s="107" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="K12" s="107" t="n">
         <v>7</v>
       </c>
       <c r="L12" s="107" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M12" s="141">
         <f>IF(B12="","",(K12+L12)/2)</f>
@@ -17647,10 +17659,10 @@
         <v>0.25</v>
       </c>
       <c r="Q12" s="107" t="n">
-        <v>1.44</v>
+        <v>1.5</v>
       </c>
       <c r="R12" s="107" t="n">
-        <v>1.5</v>
+        <v>2.06</v>
       </c>
       <c r="S12" s="141">
         <f>IF(B12="","",(Q12+R12)/2)</f>
@@ -17672,23 +17684,11 @@
         <f>IF(B12="","",O12+V12)</f>
         <v/>
       </c>
-      <c r="X12" s="142" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
-      <c r="Y12" s="353" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Z12" s="144" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AA12" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="AB12" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="X12" s="142" t="n"/>
+      <c r="Y12" s="353" t="inlineStr"/>
+      <c r="Z12" s="144" t="n"/>
+      <c r="AA12" s="144" t="n"/>
+      <c r="AB12" s="144" t="n"/>
       <c r="AC12" s="108">
         <f>IF(B12="","",IF(D12="TAPADA",(AA12+AB12)/2,0))</f>
         <v/>
@@ -17726,21 +17726,21 @@
       </c>
       <c r="D13" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E13" s="106" t="inlineStr">
         <is>
-          <t>SEC 03</t>
+          <t>SEC 04</t>
         </is>
       </c>
       <c r="F13" s="106" t="inlineStr">
         <is>
-          <t>SEC 04</t>
+          <t>SEC 07</t>
         </is>
       </c>
       <c r="G13" s="107" t="n">
-        <v>58.1</v>
+        <v>37</v>
       </c>
       <c r="H13" s="106" t="inlineStr">
         <is>
@@ -17752,10 +17752,10 @@
         <v/>
       </c>
       <c r="J13" s="107" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="K13" s="107" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L13" s="107" t="n">
         <v>9</v>
@@ -17776,10 +17776,10 @@
         <v>0.25</v>
       </c>
       <c r="Q13" s="107" t="n">
-        <v>1.5</v>
+        <v>2.06</v>
       </c>
       <c r="R13" s="107" t="n">
-        <v>2.06</v>
+        <v>2.24</v>
       </c>
       <c r="S13" s="141">
         <f>IF(B13="","",(Q13+R13)/2)</f>
@@ -17801,11 +17801,23 @@
         <f>IF(B13="","",O13+V13)</f>
         <v/>
       </c>
-      <c r="X13" s="142" t="n"/>
-      <c r="Y13" s="353" t="inlineStr"/>
-      <c r="Z13" s="144" t="n"/>
-      <c r="AA13" s="144" t="n"/>
-      <c r="AB13" s="144" t="n"/>
+      <c r="X13" s="142" t="inlineStr">
+        <is>
+          <t>3/8"</t>
+        </is>
+      </c>
+      <c r="Y13" s="353" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="Z13" s="144" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AA13" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB13" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="AC13" s="108">
         <f>IF(B13="","",IF(D13="TAPADA",(AA13+AB13)/2,0))</f>
         <v/>
@@ -17833,31 +17845,31 @@
       </c>
       <c r="B14" s="106" t="inlineStr">
         <is>
-          <t>EJE 01</t>
+          <t>EJE 02</t>
         </is>
       </c>
       <c r="C14" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D14" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E14" s="106" t="inlineStr">
         <is>
-          <t>SEC 04</t>
+          <t>SEC 09</t>
         </is>
       </c>
       <c r="F14" s="106" t="inlineStr">
         <is>
-          <t>SEC 07</t>
+          <t>SEC 10</t>
         </is>
       </c>
       <c r="G14" s="107" t="n">
-        <v>37</v>
+        <v>14.25</v>
       </c>
       <c r="H14" s="106" t="inlineStr">
         <is>
@@ -17869,13 +17881,13 @@
         <v/>
       </c>
       <c r="J14" s="107" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="K14" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="L14" s="107" t="n">
         <v>8</v>
-      </c>
-      <c r="L14" s="107" t="n">
-        <v>9</v>
       </c>
       <c r="M14" s="141">
         <f>IF(B14="","",(K14+L14)/2)</f>
@@ -17893,10 +17905,10 @@
         <v>0.25</v>
       </c>
       <c r="Q14" s="107" t="n">
-        <v>2.06</v>
+        <v>1.5</v>
       </c>
       <c r="R14" s="107" t="n">
-        <v>2.24</v>
+        <v>1.64</v>
       </c>
       <c r="S14" s="141">
         <f>IF(B14="","",(Q14+R14)/2)</f>
@@ -17918,23 +17930,11 @@
         <f>IF(B14="","",O14+V14)</f>
         <v/>
       </c>
-      <c r="X14" s="142" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
-      <c r="Y14" s="353" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Z14" s="144" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AA14" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="AB14" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="X14" s="142" t="n"/>
+      <c r="Y14" s="353" t="inlineStr"/>
+      <c r="Z14" s="144" t="n"/>
+      <c r="AA14" s="144" t="n"/>
+      <c r="AB14" s="144" t="n"/>
       <c r="AC14" s="108">
         <f>IF(B14="","",IF(D14="TAPADA",(AA14+AB14)/2,0))</f>
         <v/>
@@ -17962,7 +17962,7 @@
       </c>
       <c r="B15" s="106" t="inlineStr">
         <is>
-          <t>EJE 02</t>
+          <t>EJE 03</t>
         </is>
       </c>
       <c r="C15" s="106" t="inlineStr">
@@ -17977,16 +17977,16 @@
       </c>
       <c r="E15" s="106" t="inlineStr">
         <is>
-          <t>SEC 08</t>
+          <t>SEC 12</t>
         </is>
       </c>
       <c r="F15" s="106" t="inlineStr">
         <is>
-          <t>SEC 10</t>
+          <t>SEC 13</t>
         </is>
       </c>
       <c r="G15" s="107" t="n">
-        <v>34.25</v>
+        <v>2.4</v>
       </c>
       <c r="H15" s="106" t="inlineStr">
         <is>
@@ -18001,7 +18001,7 @@
         <v>0.2</v>
       </c>
       <c r="K15" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L15" s="107" t="n">
         <v>8</v>
@@ -18022,10 +18022,10 @@
         <v>0.25</v>
       </c>
       <c r="Q15" s="107" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R15" s="107" t="n">
-        <v>1.64</v>
+        <v>1.54</v>
       </c>
       <c r="S15" s="141">
         <f>IF(B15="","",(Q15+R15)/2)</f>
@@ -18079,7 +18079,7 @@
       </c>
       <c r="B16" s="106" t="inlineStr">
         <is>
-          <t>EJE 03</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C16" s="106" t="inlineStr">
@@ -18089,21 +18089,21 @@
       </c>
       <c r="D16" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E16" s="106" t="inlineStr">
         <is>
-          <t>SEC 11</t>
+          <t>SEC 15</t>
         </is>
       </c>
       <c r="F16" s="106" t="inlineStr">
         <is>
-          <t>SEC 13</t>
+          <t>SEC 16</t>
         </is>
       </c>
       <c r="G16" s="107" t="n">
-        <v>22.4</v>
+        <v>5.5</v>
       </c>
       <c r="H16" s="106" t="inlineStr">
         <is>
@@ -18118,10 +18118,10 @@
         <v>0.2</v>
       </c>
       <c r="K16" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L16" s="107" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M16" s="141">
         <f>IF(B16="","",(K16+L16)/2)</f>
@@ -18139,10 +18139,10 @@
         <v>0.25</v>
       </c>
       <c r="Q16" s="107" t="n">
-        <v>1.3</v>
+        <v>1.42</v>
       </c>
       <c r="R16" s="107" t="n">
-        <v>1.54</v>
+        <v>1.5</v>
       </c>
       <c r="S16" s="141">
         <f>IF(B16="","",(Q16+R16)/2)</f>
@@ -18164,11 +18164,23 @@
         <f>IF(B16="","",O16+V16)</f>
         <v/>
       </c>
-      <c r="X16" s="142" t="n"/>
-      <c r="Y16" s="353" t="inlineStr"/>
-      <c r="Z16" s="144" t="n"/>
-      <c r="AA16" s="144" t="n"/>
-      <c r="AB16" s="144" t="n"/>
+      <c r="X16" s="142" t="inlineStr">
+        <is>
+          <t>3/8"</t>
+        </is>
+      </c>
+      <c r="Y16" s="353" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="Z16" s="144" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AA16" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB16" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="AC16" s="108">
         <f>IF(B16="","",IF(D16="TAPADA",(AA16+AB16)/2,0))</f>
         <v/>
@@ -18201,7 +18213,7 @@
       </c>
       <c r="C17" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D17" s="139" t="inlineStr">
@@ -18211,16 +18223,16 @@
       </c>
       <c r="E17" s="106" t="inlineStr">
         <is>
-          <t>SEC 14</t>
+          <t>SEC 16</t>
         </is>
       </c>
       <c r="F17" s="106" t="inlineStr">
         <is>
-          <t>SEC 15</t>
+          <t>SEC 17</t>
         </is>
       </c>
       <c r="G17" s="107" t="n">
-        <v>13.65</v>
+        <v>58</v>
       </c>
       <c r="H17" s="106" t="inlineStr">
         <is>
@@ -18232,13 +18244,13 @@
         <v/>
       </c>
       <c r="J17" s="107" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="K17" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L17" s="107" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M17" s="141">
         <f>IF(B17="","",(K17+L17)/2)</f>
@@ -18256,10 +18268,10 @@
         <v>0.25</v>
       </c>
       <c r="Q17" s="107" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R17" s="107" t="n">
-        <v>1.42</v>
+        <v>2.06</v>
       </c>
       <c r="S17" s="141">
         <f>IF(B17="","",(Q17+R17)/2)</f>
@@ -18318,7 +18330,7 @@
       </c>
       <c r="C18" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 03</t>
         </is>
       </c>
       <c r="D18" s="139" t="inlineStr">
@@ -18328,16 +18340,16 @@
       </c>
       <c r="E18" s="106" t="inlineStr">
         <is>
-          <t>SEC 15</t>
+          <t>SEC 17</t>
         </is>
       </c>
       <c r="F18" s="106" t="inlineStr">
         <is>
-          <t>SEC 16</t>
+          <t>SEC 20</t>
         </is>
       </c>
       <c r="G18" s="107" t="n">
-        <v>5.5</v>
+        <v>28.55</v>
       </c>
       <c r="H18" s="106" t="inlineStr">
         <is>
@@ -18349,13 +18361,13 @@
         <v/>
       </c>
       <c r="J18" s="107" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="K18" s="107" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L18" s="107" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M18" s="141">
         <f>IF(B18="","",(K18+L18)/2)</f>
@@ -18373,10 +18385,10 @@
         <v>0.25</v>
       </c>
       <c r="Q18" s="107" t="n">
-        <v>1.42</v>
+        <v>2.06</v>
       </c>
       <c r="R18" s="107" t="n">
-        <v>1.5</v>
+        <v>2.14</v>
       </c>
       <c r="S18" s="141">
         <f>IF(B18="","",(Q18+R18)/2)</f>
@@ -18442,12 +18454,12 @@
       </c>
       <c r="B19" s="106" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C19" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 03</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D19" s="139" t="inlineStr">
@@ -18457,16 +18469,16 @@
       </c>
       <c r="E19" s="106" t="inlineStr">
         <is>
-          <t>SEC 16</t>
+          <t>SEC 22</t>
         </is>
       </c>
       <c r="F19" s="106" t="inlineStr">
         <is>
-          <t>SEC 17</t>
+          <t>SEC 23</t>
         </is>
       </c>
       <c r="G19" s="107" t="n">
-        <v>58</v>
+        <v>12.3</v>
       </c>
       <c r="H19" s="106" t="inlineStr">
         <is>
@@ -18478,13 +18490,13 @@
         <v/>
       </c>
       <c r="J19" s="107" t="n">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="K19" s="107" t="n">
         <v>7</v>
       </c>
       <c r="L19" s="107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M19" s="141">
         <f>IF(B19="","",(K19+L19)/2)</f>
@@ -18505,7 +18517,7 @@
         <v>1.5</v>
       </c>
       <c r="R19" s="107" t="n">
-        <v>2.06</v>
+        <v>1.62</v>
       </c>
       <c r="S19" s="141">
         <f>IF(B19="","",(Q19+R19)/2)</f>
@@ -18559,12 +18571,12 @@
       </c>
       <c r="B20" s="106" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C20" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
@@ -18574,16 +18586,16 @@
       </c>
       <c r="E20" s="106" t="inlineStr">
         <is>
-          <t>SEC 17</t>
+          <t>SEC 23</t>
         </is>
       </c>
       <c r="F20" s="106" t="inlineStr">
         <is>
-          <t>SEC 20</t>
+          <t>SEC 24</t>
         </is>
       </c>
       <c r="G20" s="107" t="n">
-        <v>28.55</v>
+        <v>9.9</v>
       </c>
       <c r="H20" s="106" t="inlineStr">
         <is>
@@ -18595,13 +18607,13 @@
         <v/>
       </c>
       <c r="J20" s="107" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="K20" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="L20" s="107" t="n">
         <v>8</v>
-      </c>
-      <c r="L20" s="107" t="n">
-        <v>9</v>
       </c>
       <c r="M20" s="141">
         <f>IF(B20="","",(K20+L20)/2)</f>
@@ -18619,10 +18631,10 @@
         <v>0.25</v>
       </c>
       <c r="Q20" s="107" t="n">
-        <v>2.06</v>
+        <v>1.62</v>
       </c>
       <c r="R20" s="107" t="n">
-        <v>2.14</v>
+        <v>1.72</v>
       </c>
       <c r="S20" s="141">
         <f>IF(B20="","",(Q20+R20)/2)</f>
@@ -18688,7 +18700,7 @@
       </c>
       <c r="B21" s="106" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C21" s="106" t="inlineStr">
@@ -18703,16 +18715,16 @@
       </c>
       <c r="E21" s="106" t="inlineStr">
         <is>
-          <t>SEC 21</t>
+          <t>SEC 26</t>
         </is>
       </c>
       <c r="F21" s="106" t="inlineStr">
         <is>
-          <t>SEC 23</t>
+          <t>SEC 27</t>
         </is>
       </c>
       <c r="G21" s="107" t="n">
-        <v>32.3</v>
+        <v>12.5</v>
       </c>
       <c r="H21" s="106" t="inlineStr">
         <is>
@@ -18727,7 +18739,7 @@
         <v>0.2</v>
       </c>
       <c r="K21" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L21" s="107" t="n">
         <v>8</v>
@@ -18748,7 +18760,7 @@
         <v>0.25</v>
       </c>
       <c r="Q21" s="107" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R21" s="107" t="n">
         <v>1.62</v>
@@ -18805,7 +18817,7 @@
       </c>
       <c r="B22" s="106" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C22" s="106" t="inlineStr">
@@ -18820,16 +18832,16 @@
       </c>
       <c r="E22" s="106" t="inlineStr">
         <is>
-          <t>SEC 23</t>
+          <t>SEC 27</t>
         </is>
       </c>
       <c r="F22" s="106" t="inlineStr">
         <is>
-          <t>SEC 24</t>
+          <t>SEC 30</t>
         </is>
       </c>
       <c r="G22" s="107" t="n">
-        <v>9.9</v>
+        <v>66.45</v>
       </c>
       <c r="H22" s="106" t="inlineStr">
         <is>
@@ -18847,7 +18859,7 @@
         <v>7</v>
       </c>
       <c r="L22" s="107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M22" s="141">
         <f>IF(B22="","",(K22+L22)/2)</f>
@@ -18868,7 +18880,7 @@
         <v>1.62</v>
       </c>
       <c r="R22" s="107" t="n">
-        <v>1.72</v>
+        <v>2.08</v>
       </c>
       <c r="S22" s="141">
         <f>IF(B22="","",(Q22+R22)/2)</f>
@@ -18934,7 +18946,7 @@
       </c>
       <c r="B23" s="106" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 07</t>
         </is>
       </c>
       <c r="C23" s="106" t="inlineStr">
@@ -18949,16 +18961,16 @@
       </c>
       <c r="E23" s="106" t="inlineStr">
         <is>
-          <t>SEC 25</t>
+          <t>SEC 32</t>
         </is>
       </c>
       <c r="F23" s="106" t="inlineStr">
         <is>
-          <t>SEC 27</t>
+          <t>SEC 33</t>
         </is>
       </c>
       <c r="G23" s="107" t="n">
-        <v>32.5</v>
+        <v>3.6</v>
       </c>
       <c r="H23" s="106" t="inlineStr">
         <is>
@@ -18973,7 +18985,7 @@
         <v>0.2</v>
       </c>
       <c r="K23" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L23" s="107" t="n">
         <v>8</v>
@@ -18994,10 +19006,10 @@
         <v>0.25</v>
       </c>
       <c r="Q23" s="107" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R23" s="107" t="n">
-        <v>1.62</v>
+        <v>1.52</v>
       </c>
       <c r="S23" s="141">
         <f>IF(B23="","",(Q23+R23)/2)</f>
@@ -19051,31 +19063,31 @@
       </c>
       <c r="B24" s="106" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C24" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D24" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E24" s="106" t="inlineStr">
         <is>
-          <t>SEC 27</t>
+          <t>SEC 35</t>
         </is>
       </c>
       <c r="F24" s="106" t="inlineStr">
         <is>
-          <t>SEC 30</t>
+          <t>SEC 36</t>
         </is>
       </c>
       <c r="G24" s="107" t="n">
-        <v>66.45</v>
+        <v>29.85</v>
       </c>
       <c r="H24" s="106" t="inlineStr">
         <is>
@@ -19093,7 +19105,7 @@
         <v>7</v>
       </c>
       <c r="L24" s="107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M24" s="141">
         <f>IF(B24="","",(K24+L24)/2)</f>
@@ -19111,10 +19123,10 @@
         <v>0.25</v>
       </c>
       <c r="Q24" s="107" t="n">
-        <v>1.62</v>
+        <v>1.5</v>
       </c>
       <c r="R24" s="107" t="n">
-        <v>2.08</v>
+        <v>1.8</v>
       </c>
       <c r="S24" s="141">
         <f>IF(B24="","",(Q24+R24)/2)</f>
@@ -19136,23 +19148,11 @@
         <f>IF(B24="","",O24+V24)</f>
         <v/>
       </c>
-      <c r="X24" s="142" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
-      <c r="Y24" s="353" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Z24" s="144" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AA24" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="AB24" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="X24" s="142" t="n"/>
+      <c r="Y24" s="353" t="inlineStr"/>
+      <c r="Z24" s="144" t="n"/>
+      <c r="AA24" s="144" t="n"/>
+      <c r="AB24" s="144" t="n"/>
       <c r="AC24" s="108">
         <f>IF(B24="","",IF(D24="TAPADA",(AA24+AB24)/2,0))</f>
         <v/>
@@ -19180,31 +19180,31 @@
       </c>
       <c r="B25" s="106" t="inlineStr">
         <is>
-          <t>EJE 07</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C25" s="106" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D25" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E25" s="106" t="inlineStr">
         <is>
-          <t>SEC 31</t>
+          <t>SEC 36</t>
         </is>
       </c>
       <c r="F25" s="106" t="inlineStr">
         <is>
-          <t>SEC 33</t>
+          <t>SEC 37</t>
         </is>
       </c>
       <c r="G25" s="107" t="n">
-        <v>23.6</v>
+        <v>10.85</v>
       </c>
       <c r="H25" s="106" t="inlineStr">
         <is>
@@ -19216,13 +19216,13 @@
         <v/>
       </c>
       <c r="J25" s="107" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="K25" s="107" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L25" s="107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M25" s="141">
         <f>IF(B25="","",(K25+L25)/2)</f>
@@ -19240,10 +19240,10 @@
         <v>0.25</v>
       </c>
       <c r="Q25" s="107" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="R25" s="107" t="n">
-        <v>1.52</v>
+        <v>1.9</v>
       </c>
       <c r="S25" s="141">
         <f>IF(B25="","",(Q25+R25)/2)</f>
@@ -19265,11 +19265,23 @@
         <f>IF(B25="","",O25+V25)</f>
         <v/>
       </c>
-      <c r="X25" s="142" t="n"/>
-      <c r="Y25" s="353" t="inlineStr"/>
-      <c r="Z25" s="144" t="n"/>
-      <c r="AA25" s="144" t="n"/>
-      <c r="AB25" s="144" t="n"/>
+      <c r="X25" s="142" t="inlineStr">
+        <is>
+          <t>3/8"</t>
+        </is>
+      </c>
+      <c r="Y25" s="353" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="Z25" s="144" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AA25" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB25" s="144" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="AC25" s="108">
         <f>IF(B25="","",IF(D25="TAPADA",(AA25+AB25)/2,0))</f>
         <v/>
@@ -19297,7 +19309,7 @@
       </c>
       <c r="B26" s="106" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C26" s="106" t="inlineStr">
@@ -19312,16 +19324,16 @@
       </c>
       <c r="E26" s="106" t="inlineStr">
         <is>
-          <t>SEC 34</t>
+          <t>SEC 39</t>
         </is>
       </c>
       <c r="F26" s="106" t="inlineStr">
         <is>
-          <t>SEC 36</t>
+          <t>SEC 40</t>
         </is>
       </c>
       <c r="G26" s="107" t="n">
-        <v>49.85</v>
+        <v>16</v>
       </c>
       <c r="H26" s="106" t="inlineStr">
         <is>
@@ -19333,13 +19345,13 @@
         <v/>
       </c>
       <c r="J26" s="107" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="K26" s="107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L26" s="107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M26" s="141">
         <f>IF(B26="","",(K26+L26)/2)</f>
@@ -19357,10 +19369,10 @@
         <v>0.25</v>
       </c>
       <c r="Q26" s="107" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="R26" s="107" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="S26" s="141">
         <f>IF(B26="","",(Q26+R26)/2)</f>
@@ -19414,7 +19426,7 @@
       </c>
       <c r="B27" s="106" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C27" s="106" t="inlineStr">
@@ -19429,16 +19441,16 @@
       </c>
       <c r="E27" s="106" t="inlineStr">
         <is>
-          <t>SEC 36</t>
+          <t>SEC 40</t>
         </is>
       </c>
       <c r="F27" s="106" t="inlineStr">
         <is>
-          <t>SEC 37</t>
+          <t>SEC 42</t>
         </is>
       </c>
       <c r="G27" s="107" t="n">
-        <v>10.85</v>
+        <v>6.7</v>
       </c>
       <c r="H27" s="106" t="inlineStr">
         <is>
@@ -19456,7 +19468,7 @@
         <v>8</v>
       </c>
       <c r="L27" s="107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M27" s="141">
         <f>IF(B27="","",(K27+L27)/2)</f>
@@ -19474,10 +19486,10 @@
         <v>0.25</v>
       </c>
       <c r="Q27" s="107" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="R27" s="107" t="n">
-        <v>1.9</v>
+        <v>1.82</v>
       </c>
       <c r="S27" s="141">
         <f>IF(B27="","",(Q27+R27)/2)</f>
@@ -19538,55 +19550,21 @@
       </c>
     </row>
     <row r="28" ht="36.5" customHeight="1">
-      <c r="A28" s="138" t="n">
-        <v>18</v>
-      </c>
-      <c r="B28" s="106" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C28" s="106" t="inlineStr">
-        <is>
-          <t>TRAMO 01</t>
-        </is>
-      </c>
-      <c r="D28" s="139" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-      <c r="E28" s="106" t="inlineStr">
-        <is>
-          <t>SEC 38</t>
-        </is>
-      </c>
-      <c r="F28" s="106" t="inlineStr">
-        <is>
-          <t>SEC 40</t>
-        </is>
-      </c>
-      <c r="G28" s="107" t="n">
-        <v>36</v>
-      </c>
-      <c r="H28" s="106" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
+      <c r="A28" s="138" t="n"/>
+      <c r="B28" s="106" t="n"/>
+      <c r="C28" s="106" t="n"/>
+      <c r="D28" s="139" t="n"/>
+      <c r="E28" s="106" t="n"/>
+      <c r="F28" s="106" t="n"/>
+      <c r="G28" s="107" t="n"/>
+      <c r="H28" s="106" t="n"/>
       <c r="I28" s="352">
         <f>IF(H28="","",IFERROR(VLOOKUP(H28,Listas!$A$4:$B$11,2,FALSE),""))</f>
         <v/>
       </c>
-      <c r="J28" s="107" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K28" s="107" t="n">
-        <v>6</v>
-      </c>
-      <c r="L28" s="107" t="n">
-        <v>8</v>
-      </c>
+      <c r="J28" s="107" t="n"/>
+      <c r="K28" s="107" t="n"/>
+      <c r="L28" s="107" t="n"/>
       <c r="M28" s="141">
         <f>IF(B28="","",(K28+L28)/2)</f>
         <v/>
@@ -19599,15 +19577,9 @@
         <f>IF(B28="","",N28*I28)</f>
         <v/>
       </c>
-      <c r="P28" s="107" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Q28" s="107" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R28" s="107" t="n">
-        <v>1.7</v>
-      </c>
+      <c r="P28" s="107" t="n"/>
+      <c r="Q28" s="107" t="n"/>
+      <c r="R28" s="107" t="n"/>
       <c r="S28" s="141">
         <f>IF(B28="","",(Q28+R28)/2)</f>
         <v/>
@@ -19655,55 +19627,21 @@
       </c>
     </row>
     <row r="29" ht="36.5" customHeight="1">
-      <c r="A29" s="138" t="n">
-        <v>19</v>
-      </c>
-      <c r="B29" s="106" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C29" s="106" t="inlineStr">
-        <is>
-          <t>TRAMO 02</t>
-        </is>
-      </c>
-      <c r="D29" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E29" s="106" t="inlineStr">
-        <is>
-          <t>SEC 40</t>
-        </is>
-      </c>
-      <c r="F29" s="106" t="inlineStr">
-        <is>
-          <t>SEC 42</t>
-        </is>
-      </c>
-      <c r="G29" s="107" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="H29" s="106" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
+      <c r="A29" s="138" t="n"/>
+      <c r="B29" s="106" t="n"/>
+      <c r="C29" s="106" t="n"/>
+      <c r="D29" s="139" t="n"/>
+      <c r="E29" s="106" t="n"/>
+      <c r="F29" s="106" t="n"/>
+      <c r="G29" s="107" t="n"/>
+      <c r="H29" s="106" t="n"/>
       <c r="I29" s="352">
         <f>IF(H29="","",IFERROR(VLOOKUP(H29,Listas!$A$4:$B$11,2,FALSE),""))</f>
         <v/>
       </c>
-      <c r="J29" s="107" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="K29" s="107" t="n">
-        <v>8</v>
-      </c>
-      <c r="L29" s="107" t="n">
-        <v>8</v>
-      </c>
+      <c r="J29" s="107" t="n"/>
+      <c r="K29" s="107" t="n"/>
+      <c r="L29" s="107" t="n"/>
       <c r="M29" s="141">
         <f>IF(B29="","",(K29+L29)/2)</f>
         <v/>
@@ -19716,15 +19654,9 @@
         <f>IF(B29="","",N29*I29)</f>
         <v/>
       </c>
-      <c r="P29" s="107" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Q29" s="107" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="R29" s="107" t="n">
-        <v>1.82</v>
-      </c>
+      <c r="P29" s="107" t="n"/>
+      <c r="Q29" s="107" t="n"/>
+      <c r="R29" s="107" t="n"/>
       <c r="S29" s="141">
         <f>IF(B29="","",(Q29+R29)/2)</f>
         <v/>
@@ -19745,23 +19677,11 @@
         <f>IF(B29="","",O29+V29)</f>
         <v/>
       </c>
-      <c r="X29" s="142" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
-      <c r="Y29" s="353" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Z29" s="144" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AA29" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="AB29" s="144" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="X29" s="142" t="n"/>
+      <c r="Y29" s="353" t="inlineStr"/>
+      <c r="Z29" s="144" t="n"/>
+      <c r="AA29" s="144" t="n"/>
+      <c r="AB29" s="144" t="n"/>
       <c r="AC29" s="108">
         <f>IF(B29="","",IF(D29="TAPADA",(AA29+AB29)/2,0))</f>
         <v/>
@@ -20717,20 +20637,20 @@
       </c>
       <c r="D7" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E7" s="136" t="n">
-        <v>13.2</v>
+        <v>6</v>
       </c>
       <c r="F7" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G7" s="136" t="n">
-        <v>0.3</v>
+        <v>0.37</v>
       </c>
       <c r="H7" s="136" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="I7" s="108">
         <f>IF(B7="","",(G7+H7)/2)</f>
@@ -20778,20 +20698,20 @@
       </c>
       <c r="D8" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E8" s="136" t="n">
-        <v>6</v>
+        <v>58.1</v>
       </c>
       <c r="F8" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G8" s="136" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="136" t="n">
-        <v>0.4</v>
+        <v>0.68</v>
       </c>
       <c r="I8" s="108">
         <f>IF(B8="","",(G8+H8)/2)</f>
@@ -20839,20 +20759,20 @@
       </c>
       <c r="D9" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E9" s="136" t="n">
-        <v>58.1</v>
+        <v>37</v>
       </c>
       <c r="F9" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G9" s="136" t="n">
-        <v>0.4</v>
+        <v>0.68</v>
       </c>
       <c r="H9" s="136" t="n">
-        <v>0.68</v>
+        <v>0.77</v>
       </c>
       <c r="I9" s="108">
         <f>IF(B9="","",(G9+H9)/2)</f>
@@ -20890,30 +20810,30 @@
       </c>
       <c r="B10" s="135" t="inlineStr">
         <is>
-          <t>EJE 01</t>
+          <t>EJE 02</t>
         </is>
       </c>
       <c r="C10" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D10" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>37</v>
+        <v>14.25</v>
       </c>
       <c r="F10" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G10" s="136" t="n">
-        <v>0.68</v>
+        <v>0.4</v>
       </c>
       <c r="H10" s="136" t="n">
-        <v>0.77</v>
+        <v>0.47</v>
       </c>
       <c r="I10" s="108">
         <f>IF(B10="","",(G10+H10)/2)</f>
@@ -20951,7 +20871,7 @@
       </c>
       <c r="B11" s="135" t="inlineStr">
         <is>
-          <t>EJE 02</t>
+          <t>EJE 03</t>
         </is>
       </c>
       <c r="C11" s="135" t="inlineStr">
@@ -20965,16 +20885,16 @@
         </is>
       </c>
       <c r="E11" s="136" t="n">
-        <v>34.25</v>
+        <v>2.4</v>
       </c>
       <c r="F11" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G11" s="136" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H11" s="136" t="n">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
       <c r="I11" s="108">
         <f>IF(B11="","",(G11+H11)/2)</f>
@@ -21012,7 +20932,7 @@
       </c>
       <c r="B12" s="135" t="inlineStr">
         <is>
-          <t>EJE 03</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C12" s="135" t="inlineStr">
@@ -21022,20 +20942,20 @@
       </c>
       <c r="D12" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E12" s="136" t="n">
-        <v>22.4</v>
+        <v>5.5</v>
       </c>
       <c r="F12" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G12" s="136" t="n">
-        <v>0.3</v>
+        <v>0.36</v>
       </c>
       <c r="H12" s="136" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="I12" s="108">
         <f>IF(B12="","",(G12+H12)/2)</f>
@@ -21078,7 +20998,7 @@
       </c>
       <c r="C13" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D13" s="139" t="inlineStr">
@@ -21087,16 +21007,16 @@
         </is>
       </c>
       <c r="E13" s="136" t="n">
-        <v>13.65</v>
+        <v>58</v>
       </c>
       <c r="F13" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G13" s="136" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H13" s="136" t="n">
-        <v>0.36</v>
+        <v>0.68</v>
       </c>
       <c r="I13" s="108">
         <f>IF(B13="","",(G13+H13)/2)</f>
@@ -21139,7 +21059,7 @@
       </c>
       <c r="C14" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 03</t>
         </is>
       </c>
       <c r="D14" s="139" t="inlineStr">
@@ -21148,16 +21068,16 @@
         </is>
       </c>
       <c r="E14" s="136" t="n">
-        <v>5.5</v>
+        <v>28.55</v>
       </c>
       <c r="F14" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G14" s="136" t="n">
-        <v>0.36</v>
+        <v>0.68</v>
       </c>
       <c r="H14" s="136" t="n">
-        <v>0.4</v>
+        <v>0.72</v>
       </c>
       <c r="I14" s="108">
         <f>IF(B14="","",(G14+H14)/2)</f>
@@ -21195,12 +21115,12 @@
       </c>
       <c r="B15" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C15" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 03</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D15" s="139" t="inlineStr">
@@ -21209,7 +21129,7 @@
         </is>
       </c>
       <c r="E15" s="136" t="n">
-        <v>58</v>
+        <v>12.3</v>
       </c>
       <c r="F15" s="202" t="n">
         <v>0.4</v>
@@ -21218,7 +21138,7 @@
         <v>0.4</v>
       </c>
       <c r="H15" s="136" t="n">
-        <v>0.68</v>
+        <v>0.46</v>
       </c>
       <c r="I15" s="108">
         <f>IF(B15="","",(G15+H15)/2)</f>
@@ -21256,12 +21176,12 @@
       </c>
       <c r="B16" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C16" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D16" s="139" t="inlineStr">
@@ -21270,16 +21190,16 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>28.55</v>
+        <v>9.9</v>
       </c>
       <c r="F16" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G16" s="136" t="n">
-        <v>0.68</v>
+        <v>0.46</v>
       </c>
       <c r="H16" s="136" t="n">
-        <v>0.72</v>
+        <v>0.51</v>
       </c>
       <c r="I16" s="108">
         <f>IF(B16="","",(G16+H16)/2)</f>
@@ -21317,7 +21237,7 @@
       </c>
       <c r="B17" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C17" s="135" t="inlineStr">
@@ -21331,13 +21251,13 @@
         </is>
       </c>
       <c r="E17" s="136" t="n">
-        <v>32.3</v>
+        <v>12.5</v>
       </c>
       <c r="F17" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G17" s="136" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H17" s="136" t="n">
         <v>0.46</v>
@@ -21378,7 +21298,7 @@
       </c>
       <c r="B18" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C18" s="135" t="inlineStr">
@@ -21392,7 +21312,7 @@
         </is>
       </c>
       <c r="E18" s="136" t="n">
-        <v>9.9</v>
+        <v>66.45</v>
       </c>
       <c r="F18" s="202" t="n">
         <v>0.4</v>
@@ -21401,7 +21321,7 @@
         <v>0.46</v>
       </c>
       <c r="H18" s="136" t="n">
-        <v>0.51</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I18" s="108">
         <f>IF(B18="","",(G18+H18)/2)</f>
@@ -21439,7 +21359,7 @@
       </c>
       <c r="B19" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 07</t>
         </is>
       </c>
       <c r="C19" s="135" t="inlineStr">
@@ -21453,16 +21373,16 @@
         </is>
       </c>
       <c r="E19" s="136" t="n">
-        <v>32.5</v>
+        <v>3.6</v>
       </c>
       <c r="F19" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G19" s="136" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H19" s="136" t="n">
-        <v>0.46</v>
+        <v>0.41</v>
       </c>
       <c r="I19" s="108">
         <f>IF(B19="","",(G19+H19)/2)</f>
@@ -21500,30 +21420,30 @@
       </c>
       <c r="B20" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C20" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.45</v>
+        <v>29.85</v>
       </c>
       <c r="F20" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G20" s="136" t="n">
-        <v>0.46</v>
+        <v>0.4</v>
       </c>
       <c r="H20" s="136" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="I20" s="108">
         <f>IF(B20="","",(G20+H20)/2)</f>
@@ -21561,30 +21481,30 @@
       </c>
       <c r="B21" s="135" t="inlineStr">
         <is>
-          <t>EJE 07</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C21" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D21" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E21" s="136" t="n">
-        <v>23.6</v>
+        <v>10.85</v>
       </c>
       <c r="F21" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G21" s="136" t="n">
-        <v>0.3</v>
+        <v>0.55</v>
       </c>
       <c r="H21" s="136" t="n">
-        <v>0.41</v>
+        <v>0.6</v>
       </c>
       <c r="I21" s="108">
         <f>IF(B21="","",(G21+H21)/2)</f>
@@ -21622,7 +21542,7 @@
       </c>
       <c r="B22" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C22" s="135" t="inlineStr">
@@ -21636,16 +21556,16 @@
         </is>
       </c>
       <c r="E22" s="136" t="n">
-        <v>49.85</v>
+        <v>16</v>
       </c>
       <c r="F22" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G22" s="136" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H22" s="136" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="I22" s="108">
         <f>IF(B22="","",(G22+H22)/2)</f>
@@ -21683,7 +21603,7 @@
       </c>
       <c r="B23" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C23" s="135" t="inlineStr">
@@ -21697,16 +21617,16 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.85</v>
+        <v>6.7</v>
       </c>
       <c r="F23" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G23" s="136" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="H23" s="136" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I23" s="108">
         <f>IF(B23="","",(G23+H23)/2)</f>
@@ -21739,36 +21659,14 @@
       </c>
     </row>
     <row r="24" ht="33" customHeight="1">
-      <c r="A24" s="103" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" s="135" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C24" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 01</t>
-        </is>
-      </c>
-      <c r="D24" s="139" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-      <c r="E24" s="136" t="n">
-        <v>36</v>
-      </c>
-      <c r="F24" s="202" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G24" s="136" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H24" s="136" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="A24" s="103" t="n"/>
+      <c r="B24" s="135" t="n"/>
+      <c r="C24" s="135" t="n"/>
+      <c r="D24" s="139" t="n"/>
+      <c r="E24" s="136" t="n"/>
+      <c r="F24" s="202" t="n"/>
+      <c r="G24" s="136" t="n"/>
+      <c r="H24" s="136" t="n"/>
       <c r="I24" s="108">
         <f>IF(B24="","",(G24+H24)/2)</f>
         <v/>
@@ -21800,36 +21698,14 @@
       </c>
     </row>
     <row r="25" ht="33" customHeight="1">
-      <c r="A25" s="103" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" s="135" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C25" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 02</t>
-        </is>
-      </c>
-      <c r="D25" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E25" s="136" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F25" s="202" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G25" s="136" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H25" s="136" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="A25" s="103" t="n"/>
+      <c r="B25" s="135" t="n"/>
+      <c r="C25" s="135" t="n"/>
+      <c r="D25" s="139" t="n"/>
+      <c r="E25" s="136" t="n"/>
+      <c r="F25" s="202" t="n"/>
+      <c r="G25" s="136" t="n"/>
+      <c r="H25" s="136" t="n"/>
       <c r="I25" s="108">
         <f>IF(B25="","",(G25+H25)/2)</f>
         <v/>
@@ -22547,11 +22423,11 @@
       </c>
       <c r="D7" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E7" s="136" t="n">
-        <v>13.2</v>
+        <v>6</v>
       </c>
       <c r="F7" s="176" t="n">
         <v>0</v>
@@ -22582,11 +22458,11 @@
       </c>
       <c r="D8" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E8" s="136" t="n">
-        <v>6</v>
+        <v>58.1</v>
       </c>
       <c r="F8" s="176" t="n">
         <v>0</v>
@@ -22617,11 +22493,11 @@
       </c>
       <c r="D9" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E9" s="136" t="n">
-        <v>58.1</v>
+        <v>37</v>
       </c>
       <c r="F9" s="176" t="n">
         <v>0</v>
@@ -22642,21 +22518,21 @@
       </c>
       <c r="B10" s="135" t="inlineStr">
         <is>
-          <t>EJE 01</t>
+          <t>EJE 02</t>
         </is>
       </c>
       <c r="C10" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D10" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>37</v>
+        <v>14.25</v>
       </c>
       <c r="F10" s="176" t="n">
         <v>0</v>
@@ -22677,7 +22553,7 @@
       </c>
       <c r="B11" s="135" t="inlineStr">
         <is>
-          <t>EJE 02</t>
+          <t>EJE 03</t>
         </is>
       </c>
       <c r="C11" s="135" t="inlineStr">
@@ -22691,7 +22567,7 @@
         </is>
       </c>
       <c r="E11" s="136" t="n">
-        <v>34.25</v>
+        <v>2.4</v>
       </c>
       <c r="F11" s="176" t="n">
         <v>0</v>
@@ -22712,7 +22588,7 @@
       </c>
       <c r="B12" s="135" t="inlineStr">
         <is>
-          <t>EJE 03</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C12" s="135" t="inlineStr">
@@ -22722,11 +22598,11 @@
       </c>
       <c r="D12" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E12" s="136" t="n">
-        <v>22.4</v>
+        <v>5.5</v>
       </c>
       <c r="F12" s="176" t="n">
         <v>0</v>
@@ -22752,7 +22628,7 @@
       </c>
       <c r="C13" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D13" s="139" t="inlineStr">
@@ -22761,7 +22637,7 @@
         </is>
       </c>
       <c r="E13" s="136" t="n">
-        <v>13.65</v>
+        <v>58</v>
       </c>
       <c r="F13" s="176" t="n">
         <v>0</v>
@@ -22787,7 +22663,7 @@
       </c>
       <c r="C14" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 03</t>
         </is>
       </c>
       <c r="D14" s="139" t="inlineStr">
@@ -22796,7 +22672,7 @@
         </is>
       </c>
       <c r="E14" s="136" t="n">
-        <v>5.5</v>
+        <v>28.55</v>
       </c>
       <c r="F14" s="176" t="n">
         <v>0</v>
@@ -22817,12 +22693,12 @@
       </c>
       <c r="B15" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C15" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 03</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D15" s="139" t="inlineStr">
@@ -22831,7 +22707,7 @@
         </is>
       </c>
       <c r="E15" s="136" t="n">
-        <v>58</v>
+        <v>12.3</v>
       </c>
       <c r="F15" s="176" t="n">
         <v>0</v>
@@ -22852,12 +22728,12 @@
       </c>
       <c r="B16" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C16" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 04</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D16" s="139" t="inlineStr">
@@ -22866,7 +22742,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>28.55</v>
+        <v>9.9</v>
       </c>
       <c r="F16" s="176" t="n">
         <v>0</v>
@@ -22887,7 +22763,7 @@
       </c>
       <c r="B17" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C17" s="135" t="inlineStr">
@@ -22901,7 +22777,7 @@
         </is>
       </c>
       <c r="E17" s="136" t="n">
-        <v>32.3</v>
+        <v>12.5</v>
       </c>
       <c r="F17" s="176" t="n">
         <v>0</v>
@@ -22922,7 +22798,7 @@
       </c>
       <c r="B18" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C18" s="135" t="inlineStr">
@@ -22936,7 +22812,7 @@
         </is>
       </c>
       <c r="E18" s="136" t="n">
-        <v>9.9</v>
+        <v>66.45</v>
       </c>
       <c r="F18" s="176" t="n">
         <v>0</v>
@@ -22957,7 +22833,7 @@
       </c>
       <c r="B19" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 07</t>
         </is>
       </c>
       <c r="C19" s="135" t="inlineStr">
@@ -22971,7 +22847,7 @@
         </is>
       </c>
       <c r="E19" s="136" t="n">
-        <v>32.5</v>
+        <v>3.6</v>
       </c>
       <c r="F19" s="176" t="n">
         <v>0</v>
@@ -22992,21 +22868,21 @@
       </c>
       <c r="B20" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C20" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.45</v>
+        <v>29.85</v>
       </c>
       <c r="F20" s="176" t="n">
         <v>0</v>
@@ -23027,21 +22903,21 @@
       </c>
       <c r="B21" s="135" t="inlineStr">
         <is>
-          <t>EJE 07</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C21" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D21" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E21" s="136" t="n">
-        <v>23.6</v>
+        <v>10.85</v>
       </c>
       <c r="F21" s="176" t="n">
         <v>0</v>
@@ -23062,7 +22938,7 @@
       </c>
       <c r="B22" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C22" s="135" t="inlineStr">
@@ -23076,7 +22952,7 @@
         </is>
       </c>
       <c r="E22" s="136" t="n">
-        <v>49.85</v>
+        <v>16</v>
       </c>
       <c r="F22" s="176" t="n">
         <v>0</v>
@@ -23097,7 +22973,7 @@
       </c>
       <c r="B23" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 09</t>
         </is>
       </c>
       <c r="C23" s="135" t="inlineStr">
@@ -23111,7 +22987,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.85</v>
+        <v>6.7</v>
       </c>
       <c r="F23" s="176" t="n">
         <v>0</v>
@@ -23127,30 +23003,12 @@
       </c>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="103" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" s="135" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C24" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 01</t>
-        </is>
-      </c>
-      <c r="D24" s="139" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-      <c r="E24" s="136" t="n">
-        <v>36</v>
-      </c>
-      <c r="F24" s="176" t="n">
-        <v>0</v>
-      </c>
+      <c r="A24" s="103" t="n"/>
+      <c r="B24" s="135" t="n"/>
+      <c r="C24" s="135" t="n"/>
+      <c r="D24" s="139" t="n"/>
+      <c r="E24" s="136" t="n"/>
+      <c r="F24" s="176" t="n"/>
       <c r="G24" s="177">
         <f>IF(B24="","",IF(D24="ABIERTA",IF(E24-F24&lt;0,0,E24-F24),0))</f>
         <v/>
@@ -23162,30 +23020,12 @@
       </c>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="103" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" s="135" t="inlineStr">
-        <is>
-          <t>EJE 09</t>
-        </is>
-      </c>
-      <c r="C25" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 02</t>
-        </is>
-      </c>
-      <c r="D25" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E25" s="136" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F25" s="176" t="n">
-        <v>0</v>
-      </c>
+      <c r="A25" s="103" t="n"/>
+      <c r="B25" s="135" t="n"/>
+      <c r="C25" s="135" t="n"/>
+      <c r="D25" s="139" t="n"/>
+      <c r="E25" s="136" t="n"/>
+      <c r="F25" s="176" t="n"/>
       <c r="G25" s="177">
         <f>IF(B25="","",IF(D25="ABIERTA",IF(E25-F25&lt;0,0,E25-F25),0))</f>
         <v/>

</xml_diff>

<commit_message>
Metrado Varones: curado y rejillas con todos los tramos; filas sobrantes de la plantilla limpiadas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
@@ -20637,20 +20637,20 @@
       </c>
       <c r="D7" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E7" s="136" t="n">
-        <v>6</v>
+        <v>13.2</v>
       </c>
       <c r="F7" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G7" s="136" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H7" s="136" t="n">
         <v>0.37</v>
-      </c>
-      <c r="H7" s="136" t="n">
-        <v>0.4</v>
       </c>
       <c r="I7" s="108">
         <f>IF(B7="","",(G7+H7)/2)</f>
@@ -20698,20 +20698,20 @@
       </c>
       <c r="D8" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E8" s="136" t="n">
-        <v>58.1</v>
+        <v>6</v>
       </c>
       <c r="F8" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G8" s="136" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="H8" s="136" t="n">
         <v>0.4</v>
-      </c>
-      <c r="H8" s="136" t="n">
-        <v>0.68</v>
       </c>
       <c r="I8" s="108">
         <f>IF(B8="","",(G8+H8)/2)</f>
@@ -20759,20 +20759,20 @@
       </c>
       <c r="D9" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E9" s="136" t="n">
-        <v>37</v>
+        <v>58.1</v>
       </c>
       <c r="F9" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G9" s="136" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H9" s="136" t="n">
         <v>0.68</v>
-      </c>
-      <c r="H9" s="136" t="n">
-        <v>0.77</v>
       </c>
       <c r="I9" s="108">
         <f>IF(B9="","",(G9+H9)/2)</f>
@@ -20810,30 +20810,30 @@
       </c>
       <c r="B10" s="135" t="inlineStr">
         <is>
-          <t>EJE 02</t>
+          <t>EJE 01</t>
         </is>
       </c>
       <c r="C10" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 04</t>
         </is>
       </c>
       <c r="D10" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>14.25</v>
+        <v>37</v>
       </c>
       <c r="F10" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G10" s="136" t="n">
-        <v>0.4</v>
+        <v>0.68</v>
       </c>
       <c r="H10" s="136" t="n">
-        <v>0.47</v>
+        <v>0.77</v>
       </c>
       <c r="I10" s="108">
         <f>IF(B10="","",(G10+H10)/2)</f>
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B11" s="135" t="inlineStr">
         <is>
-          <t>EJE 03</t>
+          <t>EJE 02</t>
         </is>
       </c>
       <c r="C11" s="135" t="inlineStr">
@@ -20885,16 +20885,16 @@
         </is>
       </c>
       <c r="E11" s="136" t="n">
-        <v>2.4</v>
+        <v>34.25</v>
       </c>
       <c r="F11" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G11" s="136" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H11" s="136" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="I11" s="108">
         <f>IF(B11="","",(G11+H11)/2)</f>
@@ -20932,7 +20932,7 @@
       </c>
       <c r="B12" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 03</t>
         </is>
       </c>
       <c r="C12" s="135" t="inlineStr">
@@ -20942,20 +20942,20 @@
       </c>
       <c r="D12" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E12" s="136" t="n">
-        <v>5.5</v>
+        <v>22.4</v>
       </c>
       <c r="F12" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G12" s="136" t="n">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="H12" s="136" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="I12" s="108">
         <f>IF(B12="","",(G12+H12)/2)</f>
@@ -20998,7 +20998,7 @@
       </c>
       <c r="C13" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D13" s="139" t="inlineStr">
@@ -21007,16 +21007,16 @@
         </is>
       </c>
       <c r="E13" s="136" t="n">
-        <v>58</v>
+        <v>13.65</v>
       </c>
       <c r="F13" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G13" s="136" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H13" s="136" t="n">
-        <v>0.68</v>
+        <v>0.36</v>
       </c>
       <c r="I13" s="108">
         <f>IF(B13="","",(G13+H13)/2)</f>
@@ -21059,7 +21059,7 @@
       </c>
       <c r="C14" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 03</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D14" s="139" t="inlineStr">
@@ -21068,16 +21068,16 @@
         </is>
       </c>
       <c r="E14" s="136" t="n">
-        <v>28.55</v>
+        <v>5.5</v>
       </c>
       <c r="F14" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G14" s="136" t="n">
-        <v>0.68</v>
+        <v>0.36</v>
       </c>
       <c r="H14" s="136" t="n">
-        <v>0.72</v>
+        <v>0.4</v>
       </c>
       <c r="I14" s="108">
         <f>IF(B14="","",(G14+H14)/2)</f>
@@ -21115,12 +21115,12 @@
       </c>
       <c r="B15" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C15" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 03</t>
         </is>
       </c>
       <c r="D15" s="139" t="inlineStr">
@@ -21129,7 +21129,7 @@
         </is>
       </c>
       <c r="E15" s="136" t="n">
-        <v>12.3</v>
+        <v>58</v>
       </c>
       <c r="F15" s="202" t="n">
         <v>0.4</v>
@@ -21138,7 +21138,7 @@
         <v>0.4</v>
       </c>
       <c r="H15" s="136" t="n">
-        <v>0.46</v>
+        <v>0.68</v>
       </c>
       <c r="I15" s="108">
         <f>IF(B15="","",(G15+H15)/2)</f>
@@ -21176,12 +21176,12 @@
       </c>
       <c r="B16" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C16" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 04</t>
         </is>
       </c>
       <c r="D16" s="139" t="inlineStr">
@@ -21190,16 +21190,16 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>9.9</v>
+        <v>28.55</v>
       </c>
       <c r="F16" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G16" s="136" t="n">
-        <v>0.46</v>
+        <v>0.68</v>
       </c>
       <c r="H16" s="136" t="n">
-        <v>0.51</v>
+        <v>0.72</v>
       </c>
       <c r="I16" s="108">
         <f>IF(B16="","",(G16+H16)/2)</f>
@@ -21237,7 +21237,7 @@
       </c>
       <c r="B17" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C17" s="135" t="inlineStr">
@@ -21251,13 +21251,13 @@
         </is>
       </c>
       <c r="E17" s="136" t="n">
-        <v>12.5</v>
+        <v>32.3</v>
       </c>
       <c r="F17" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G17" s="136" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H17" s="136" t="n">
         <v>0.46</v>
@@ -21298,7 +21298,7 @@
       </c>
       <c r="B18" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C18" s="135" t="inlineStr">
@@ -21312,7 +21312,7 @@
         </is>
       </c>
       <c r="E18" s="136" t="n">
-        <v>66.45</v>
+        <v>9.9</v>
       </c>
       <c r="F18" s="202" t="n">
         <v>0.4</v>
@@ -21321,7 +21321,7 @@
         <v>0.46</v>
       </c>
       <c r="H18" s="136" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.51</v>
       </c>
       <c r="I18" s="108">
         <f>IF(B18="","",(G18+H18)/2)</f>
@@ -21359,7 +21359,7 @@
       </c>
       <c r="B19" s="135" t="inlineStr">
         <is>
-          <t>EJE 07</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C19" s="135" t="inlineStr">
@@ -21373,16 +21373,16 @@
         </is>
       </c>
       <c r="E19" s="136" t="n">
-        <v>3.6</v>
+        <v>32.5</v>
       </c>
       <c r="F19" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G19" s="136" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H19" s="136" t="n">
-        <v>0.41</v>
+        <v>0.46</v>
       </c>
       <c r="I19" s="108">
         <f>IF(B19="","",(G19+H19)/2)</f>
@@ -21420,30 +21420,30 @@
       </c>
       <c r="B20" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C20" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>29.85</v>
+        <v>66.45</v>
       </c>
       <c r="F20" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G20" s="136" t="n">
-        <v>0.4</v>
+        <v>0.46</v>
       </c>
       <c r="H20" s="136" t="n">
-        <v>0.55</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I20" s="108">
         <f>IF(B20="","",(G20+H20)/2)</f>
@@ -21481,30 +21481,30 @@
       </c>
       <c r="B21" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 07</t>
         </is>
       </c>
       <c r="C21" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D21" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E21" s="136" t="n">
-        <v>10.85</v>
+        <v>23.6</v>
       </c>
       <c r="F21" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G21" s="136" t="n">
-        <v>0.55</v>
+        <v>0.3</v>
       </c>
       <c r="H21" s="136" t="n">
-        <v>0.6</v>
+        <v>0.41</v>
       </c>
       <c r="I21" s="108">
         <f>IF(B21="","",(G21+H21)/2)</f>
@@ -21542,7 +21542,7 @@
       </c>
       <c r="B22" s="135" t="inlineStr">
         <is>
-          <t>EJE 09</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C22" s="135" t="inlineStr">
@@ -21556,16 +21556,16 @@
         </is>
       </c>
       <c r="E22" s="136" t="n">
-        <v>16</v>
+        <v>49.85</v>
       </c>
       <c r="F22" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G22" s="136" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H22" s="136" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="I22" s="108">
         <f>IF(B22="","",(G22+H22)/2)</f>
@@ -21603,7 +21603,7 @@
       </c>
       <c r="B23" s="135" t="inlineStr">
         <is>
-          <t>EJE 09</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C23" s="135" t="inlineStr">
@@ -21617,16 +21617,16 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>6.7</v>
+        <v>10.85</v>
       </c>
       <c r="F23" s="202" t="n">
         <v>0.4</v>
       </c>
       <c r="G23" s="136" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="H23" s="136" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="I23" s="108">
         <f>IF(B23="","",(G23+H23)/2)</f>
@@ -21659,14 +21659,36 @@
       </c>
     </row>
     <row r="24" ht="33" customHeight="1">
-      <c r="A24" s="103" t="n"/>
-      <c r="B24" s="135" t="n"/>
-      <c r="C24" s="135" t="n"/>
-      <c r="D24" s="139" t="n"/>
-      <c r="E24" s="136" t="n"/>
-      <c r="F24" s="202" t="n"/>
-      <c r="G24" s="136" t="n"/>
-      <c r="H24" s="136" t="n"/>
+      <c r="A24" s="103" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="135" t="inlineStr">
+        <is>
+          <t>EJE 09</t>
+        </is>
+      </c>
+      <c r="C24" s="135" t="inlineStr">
+        <is>
+          <t>TRAMO 01</t>
+        </is>
+      </c>
+      <c r="D24" s="139" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="E24" s="136" t="n">
+        <v>36</v>
+      </c>
+      <c r="F24" s="202" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G24" s="136" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H24" s="136" t="n">
+        <v>0.5</v>
+      </c>
       <c r="I24" s="108">
         <f>IF(B24="","",(G24+H24)/2)</f>
         <v/>
@@ -21698,14 +21720,36 @@
       </c>
     </row>
     <row r="25" ht="33" customHeight="1">
-      <c r="A25" s="103" t="n"/>
-      <c r="B25" s="135" t="n"/>
-      <c r="C25" s="135" t="n"/>
-      <c r="D25" s="139" t="n"/>
-      <c r="E25" s="136" t="n"/>
-      <c r="F25" s="202" t="n"/>
-      <c r="G25" s="136" t="n"/>
-      <c r="H25" s="136" t="n"/>
+      <c r="A25" s="103" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="135" t="inlineStr">
+        <is>
+          <t>EJE 09</t>
+        </is>
+      </c>
+      <c r="C25" s="135" t="inlineStr">
+        <is>
+          <t>TRAMO 02</t>
+        </is>
+      </c>
+      <c r="D25" s="139" t="inlineStr">
+        <is>
+          <t>TAPADA</t>
+        </is>
+      </c>
+      <c r="E25" s="136" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F25" s="202" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G25" s="136" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H25" s="136" t="n">
+        <v>0.5600000000000001</v>
+      </c>
       <c r="I25" s="108">
         <f>IF(B25="","",(G25+H25)/2)</f>
         <v/>
@@ -22049,36 +22093,14 @@
       </c>
     </row>
     <row r="34" ht="33" customHeight="1">
-      <c r="A34" s="103" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="135" t="inlineStr">
-        <is>
-          <t>EJE 11</t>
-        </is>
-      </c>
-      <c r="C34" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 03</t>
-        </is>
-      </c>
-      <c r="D34" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E34" s="136" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F34" s="202" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G34" s="136" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="H34" s="136" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="A34" s="103" t="n"/>
+      <c r="B34" s="135" t="n"/>
+      <c r="C34" s="135" t="n"/>
+      <c r="D34" s="139" t="n"/>
+      <c r="E34" s="136" t="n"/>
+      <c r="F34" s="202" t="n"/>
+      <c r="G34" s="136" t="n"/>
+      <c r="H34" s="136" t="n"/>
       <c r="I34" s="108">
         <f>IF(B34="","",(G34+H34)/2)</f>
         <v/>
@@ -22110,36 +22132,14 @@
       </c>
     </row>
     <row r="35" ht="33" customHeight="1">
-      <c r="A35" s="103" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" s="135" t="inlineStr">
-        <is>
-          <t>EJE 12</t>
-        </is>
-      </c>
-      <c r="C35" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 01</t>
-        </is>
-      </c>
-      <c r="D35" s="139" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-      <c r="E35" s="136" t="n">
-        <v>52.47</v>
-      </c>
-      <c r="F35" s="202" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G35" s="136" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H35" s="136" t="n">
-        <v>0.5600000000000001</v>
-      </c>
+      <c r="A35" s="103" t="n"/>
+      <c r="B35" s="135" t="n"/>
+      <c r="C35" s="135" t="n"/>
+      <c r="D35" s="139" t="n"/>
+      <c r="E35" s="136" t="n"/>
+      <c r="F35" s="202" t="n"/>
+      <c r="G35" s="136" t="n"/>
+      <c r="H35" s="136" t="n"/>
       <c r="I35" s="108">
         <f>IF(B35="","",(G35+H35)/2)</f>
         <v/>
@@ -22171,36 +22171,14 @@
       </c>
     </row>
     <row r="36" ht="33" customHeight="1">
-      <c r="A36" s="103" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" s="135" t="inlineStr">
-        <is>
-          <t>EJE 12</t>
-        </is>
-      </c>
-      <c r="C36" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 02</t>
-        </is>
-      </c>
-      <c r="D36" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E36" s="136" t="n">
-        <v>56.64</v>
-      </c>
-      <c r="F36" s="202" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G36" s="136" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="H36" s="136" t="n">
-        <v>0.8</v>
-      </c>
+      <c r="A36" s="103" t="n"/>
+      <c r="B36" s="135" t="n"/>
+      <c r="C36" s="135" t="n"/>
+      <c r="D36" s="139" t="n"/>
+      <c r="E36" s="136" t="n"/>
+      <c r="F36" s="202" t="n"/>
+      <c r="G36" s="136" t="n"/>
+      <c r="H36" s="136" t="n"/>
       <c r="I36" s="108">
         <f>IF(B36="","",(G36+H36)/2)</f>
         <v/>
@@ -22423,11 +22401,11 @@
       </c>
       <c r="D7" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E7" s="136" t="n">
-        <v>6</v>
+        <v>13.2</v>
       </c>
       <c r="F7" s="176" t="n">
         <v>0</v>
@@ -22458,11 +22436,11 @@
       </c>
       <c r="D8" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E8" s="136" t="n">
-        <v>58.1</v>
+        <v>6</v>
       </c>
       <c r="F8" s="176" t="n">
         <v>0</v>
@@ -22493,11 +22471,11 @@
       </c>
       <c r="D9" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E9" s="136" t="n">
-        <v>37</v>
+        <v>58.1</v>
       </c>
       <c r="F9" s="176" t="n">
         <v>0</v>
@@ -22518,21 +22496,21 @@
       </c>
       <c r="B10" s="135" t="inlineStr">
         <is>
-          <t>EJE 02</t>
+          <t>EJE 01</t>
         </is>
       </c>
       <c r="C10" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 04</t>
         </is>
       </c>
       <c r="D10" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>14.25</v>
+        <v>37</v>
       </c>
       <c r="F10" s="176" t="n">
         <v>0</v>
@@ -22553,7 +22531,7 @@
       </c>
       <c r="B11" s="135" t="inlineStr">
         <is>
-          <t>EJE 03</t>
+          <t>EJE 02</t>
         </is>
       </c>
       <c r="C11" s="135" t="inlineStr">
@@ -22567,7 +22545,7 @@
         </is>
       </c>
       <c r="E11" s="136" t="n">
-        <v>2.4</v>
+        <v>34.25</v>
       </c>
       <c r="F11" s="176" t="n">
         <v>0</v>
@@ -22588,7 +22566,7 @@
       </c>
       <c r="B12" s="135" t="inlineStr">
         <is>
-          <t>EJE 04</t>
+          <t>EJE 03</t>
         </is>
       </c>
       <c r="C12" s="135" t="inlineStr">
@@ -22598,11 +22576,11 @@
       </c>
       <c r="D12" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E12" s="136" t="n">
-        <v>5.5</v>
+        <v>22.4</v>
       </c>
       <c r="F12" s="176" t="n">
         <v>0</v>
@@ -22628,7 +22606,7 @@
       </c>
       <c r="C13" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D13" s="139" t="inlineStr">
@@ -22637,7 +22615,7 @@
         </is>
       </c>
       <c r="E13" s="136" t="n">
-        <v>58</v>
+        <v>13.65</v>
       </c>
       <c r="F13" s="176" t="n">
         <v>0</v>
@@ -22663,7 +22641,7 @@
       </c>
       <c r="C14" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 03</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D14" s="139" t="inlineStr">
@@ -22672,7 +22650,7 @@
         </is>
       </c>
       <c r="E14" s="136" t="n">
-        <v>28.55</v>
+        <v>5.5</v>
       </c>
       <c r="F14" s="176" t="n">
         <v>0</v>
@@ -22693,12 +22671,12 @@
       </c>
       <c r="B15" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C15" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 03</t>
         </is>
       </c>
       <c r="D15" s="139" t="inlineStr">
@@ -22707,7 +22685,7 @@
         </is>
       </c>
       <c r="E15" s="136" t="n">
-        <v>12.3</v>
+        <v>58</v>
       </c>
       <c r="F15" s="176" t="n">
         <v>0</v>
@@ -22728,12 +22706,12 @@
       </c>
       <c r="B16" s="135" t="inlineStr">
         <is>
-          <t>EJE 05</t>
+          <t>EJE 04</t>
         </is>
       </c>
       <c r="C16" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 04</t>
         </is>
       </c>
       <c r="D16" s="139" t="inlineStr">
@@ -22742,7 +22720,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>9.9</v>
+        <v>28.55</v>
       </c>
       <c r="F16" s="176" t="n">
         <v>0</v>
@@ -22763,7 +22741,7 @@
       </c>
       <c r="B17" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C17" s="135" t="inlineStr">
@@ -22777,7 +22755,7 @@
         </is>
       </c>
       <c r="E17" s="136" t="n">
-        <v>12.5</v>
+        <v>32.3</v>
       </c>
       <c r="F17" s="176" t="n">
         <v>0</v>
@@ -22798,7 +22776,7 @@
       </c>
       <c r="B18" s="135" t="inlineStr">
         <is>
-          <t>EJE 06</t>
+          <t>EJE 05</t>
         </is>
       </c>
       <c r="C18" s="135" t="inlineStr">
@@ -22812,7 +22790,7 @@
         </is>
       </c>
       <c r="E18" s="136" t="n">
-        <v>66.45</v>
+        <v>9.9</v>
       </c>
       <c r="F18" s="176" t="n">
         <v>0</v>
@@ -22833,7 +22811,7 @@
       </c>
       <c r="B19" s="135" t="inlineStr">
         <is>
-          <t>EJE 07</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C19" s="135" t="inlineStr">
@@ -22847,7 +22825,7 @@
         </is>
       </c>
       <c r="E19" s="136" t="n">
-        <v>3.6</v>
+        <v>32.5</v>
       </c>
       <c r="F19" s="176" t="n">
         <v>0</v>
@@ -22868,21 +22846,21 @@
       </c>
       <c r="B20" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 06</t>
         </is>
       </c>
       <c r="C20" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 01</t>
+          <t>TRAMO 02</t>
         </is>
       </c>
       <c r="D20" s="139" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>TAPADA</t>
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>29.85</v>
+        <v>66.45</v>
       </c>
       <c r="F20" s="176" t="n">
         <v>0</v>
@@ -22903,21 +22881,21 @@
       </c>
       <c r="B21" s="135" t="inlineStr">
         <is>
-          <t>EJE 08</t>
+          <t>EJE 07</t>
         </is>
       </c>
       <c r="C21" s="135" t="inlineStr">
         <is>
-          <t>TRAMO 02</t>
+          <t>TRAMO 01</t>
         </is>
       </c>
       <c r="D21" s="139" t="inlineStr">
         <is>
-          <t>TAPADA</t>
+          <t>ABIERTA</t>
         </is>
       </c>
       <c r="E21" s="136" t="n">
-        <v>10.85</v>
+        <v>23.6</v>
       </c>
       <c r="F21" s="176" t="n">
         <v>0</v>
@@ -22938,7 +22916,7 @@
       </c>
       <c r="B22" s="135" t="inlineStr">
         <is>
-          <t>EJE 09</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C22" s="135" t="inlineStr">
@@ -22952,7 +22930,7 @@
         </is>
       </c>
       <c r="E22" s="136" t="n">
-        <v>16</v>
+        <v>49.85</v>
       </c>
       <c r="F22" s="176" t="n">
         <v>0</v>
@@ -22973,7 +22951,7 @@
       </c>
       <c r="B23" s="135" t="inlineStr">
         <is>
-          <t>EJE 09</t>
+          <t>EJE 08</t>
         </is>
       </c>
       <c r="C23" s="135" t="inlineStr">
@@ -22987,7 +22965,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>6.7</v>
+        <v>10.85</v>
       </c>
       <c r="F23" s="176" t="n">
         <v>0</v>
@@ -23003,12 +22981,30 @@
       </c>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="103" t="n"/>
-      <c r="B24" s="135" t="n"/>
-      <c r="C24" s="135" t="n"/>
-      <c r="D24" s="139" t="n"/>
-      <c r="E24" s="136" t="n"/>
-      <c r="F24" s="176" t="n"/>
+      <c r="A24" s="103" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="135" t="inlineStr">
+        <is>
+          <t>EJE 09</t>
+        </is>
+      </c>
+      <c r="C24" s="135" t="inlineStr">
+        <is>
+          <t>TRAMO 01</t>
+        </is>
+      </c>
+      <c r="D24" s="139" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="E24" s="136" t="n">
+        <v>36</v>
+      </c>
+      <c r="F24" s="176" t="n">
+        <v>0</v>
+      </c>
       <c r="G24" s="177">
         <f>IF(B24="","",IF(D24="ABIERTA",IF(E24-F24&lt;0,0,E24-F24),0))</f>
         <v/>
@@ -23020,12 +23016,30 @@
       </c>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="103" t="n"/>
-      <c r="B25" s="135" t="n"/>
-      <c r="C25" s="135" t="n"/>
-      <c r="D25" s="139" t="n"/>
-      <c r="E25" s="136" t="n"/>
-      <c r="F25" s="176" t="n"/>
+      <c r="A25" s="103" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="135" t="inlineStr">
+        <is>
+          <t>EJE 09</t>
+        </is>
+      </c>
+      <c r="C25" s="135" t="inlineStr">
+        <is>
+          <t>TRAMO 02</t>
+        </is>
+      </c>
+      <c r="D25" s="139" t="inlineStr">
+        <is>
+          <t>TAPADA</t>
+        </is>
+      </c>
+      <c r="E25" s="136" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F25" s="176" t="n">
+        <v>0</v>
+      </c>
       <c r="G25" s="177">
         <f>IF(B25="","",IF(D25="ABIERTA",IF(E25-F25&lt;0,0,E25-F25),0))</f>
         <v/>
@@ -23173,30 +23187,12 @@
       </c>
     </row>
     <row r="34" ht="27" customHeight="1">
-      <c r="A34" s="103" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="135" t="inlineStr">
-        <is>
-          <t>EJE 11</t>
-        </is>
-      </c>
-      <c r="C34" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 03</t>
-        </is>
-      </c>
-      <c r="D34" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E34" s="136" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F34" s="176" t="n">
-        <v>0</v>
-      </c>
+      <c r="A34" s="103" t="n"/>
+      <c r="B34" s="135" t="n"/>
+      <c r="C34" s="135" t="n"/>
+      <c r="D34" s="139" t="n"/>
+      <c r="E34" s="136" t="n"/>
+      <c r="F34" s="176" t="n"/>
       <c r="G34" s="177">
         <f>IF(B34="","",IF(D34="ABIERTA",IF(E34-F34&lt;0,0,E34-F34),0))</f>
         <v/>
@@ -23208,30 +23204,12 @@
       </c>
     </row>
     <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="103" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" s="135" t="inlineStr">
-        <is>
-          <t>EJE 12</t>
-        </is>
-      </c>
-      <c r="C35" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 01</t>
-        </is>
-      </c>
-      <c r="D35" s="139" t="inlineStr">
-        <is>
-          <t>ABIERTA</t>
-        </is>
-      </c>
-      <c r="E35" s="136" t="n">
-        <v>52.47</v>
-      </c>
-      <c r="F35" s="176" t="n">
-        <v>0</v>
-      </c>
+      <c r="A35" s="103" t="n"/>
+      <c r="B35" s="135" t="n"/>
+      <c r="C35" s="135" t="n"/>
+      <c r="D35" s="139" t="n"/>
+      <c r="E35" s="136" t="n"/>
+      <c r="F35" s="176" t="n"/>
       <c r="G35" s="177">
         <f>IF(B35="","",IF(D35="ABIERTA",IF(E35-F35&lt;0,0,E35-F35),0))</f>
         <v/>
@@ -23243,30 +23221,12 @@
       </c>
     </row>
     <row r="36" ht="27" customHeight="1">
-      <c r="A36" s="103" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" s="135" t="inlineStr">
-        <is>
-          <t>EJE 12</t>
-        </is>
-      </c>
-      <c r="C36" s="135" t="inlineStr">
-        <is>
-          <t>TRAMO 02</t>
-        </is>
-      </c>
-      <c r="D36" s="139" t="inlineStr">
-        <is>
-          <t>TAPADA</t>
-        </is>
-      </c>
-      <c r="E36" s="136" t="n">
-        <v>56.64</v>
-      </c>
-      <c r="F36" s="176" t="n">
-        <v>0</v>
-      </c>
+      <c r="A36" s="103" t="n"/>
+      <c r="B36" s="135" t="n"/>
+      <c r="C36" s="135" t="n"/>
+      <c r="D36" s="139" t="n"/>
+      <c r="E36" s="136" t="n"/>
+      <c r="F36" s="176" t="n"/>
       <c r="G36" s="177">
         <f>IF(B36="","",IF(D36="ABIERTA",IF(E36-F36&lt;0,0,E36-F36),0))</f>
         <v/>

</xml_diff>

<commit_message>
CAR Varones: memoria de calculo Excel, metrado del colector sobre la planilla de cunetas y acortamiento de cunetas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
@@ -17,8 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METRADO DE REJILLAS" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METRADO JUNTA DE DILATACION" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLANILLA TAPAS REGISTRO INTERNO" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARAMETROS" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="13" state="hidden" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CUNETAS - LLEGADA AL COLECTOR" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARAMETROS" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="14" state="hidden" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMEN'!$A$1:$D$49</definedName>
@@ -40,7 +41,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="48">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -295,8 +296,47 @@
       <color rgb="FF1F4E78"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial Narrow"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -508,8 +548,28 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="50">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -1122,6 +1182,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1129,7 +1195,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="361">
+  <cellXfs count="374">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2130,6 +2196,41 @@
     </xf>
     <xf numFmtId="165" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="39" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="40" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="39" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="45" fillId="41" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="45" fillId="42" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2826,7 +2927,7 @@
       </c>
       <c r="B5" s="205" t="inlineStr">
         <is>
-          <t>CENTRO DE ACOGIDA RESIDENCIAL (CAR) VARONES - DISTRITO DE MORALES, PROVINCIA Y DEPARTAMENTO DE SAN MARTIN, con CUI N.° 2705619</t>
+          <t>CREACIÓN DEL SERVICIO DE PROTECCIÓN INTEGRAL A NIÑAS, NIÑOS Y ADOLESCENTES SIN CUIDADOS PARENTALES O EN RIESGO DE PERDERLOS EN CENTRO DE ACOGIDA RESIDENCIAL - VARONES DISTRITO DE MORALES DE LA PROVINCIA DE SAN MARTÍN DEL DEPARTAMENTO DE SAN MARTÍN, con CUI N.° 2705619</t>
         </is>
       </c>
       <c r="C5" s="313" t="n"/>
@@ -3924,7 +4025,7 @@
       </c>
       <c r="C13" s="184" t="n"/>
       <c r="D13" s="190" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E13" s="188">
         <f>+'CONCRETO EN CUNETAS'!E10</f>
@@ -4038,7 +4139,7 @@
       </c>
       <c r="C16" s="184" t="n"/>
       <c r="D16" s="190" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E16" s="188">
         <f>+'CONCRETO EN CUNETAS'!E46</f>
@@ -4114,7 +4215,7 @@
       </c>
       <c r="C18" s="184" t="n"/>
       <c r="D18" s="190" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E18" s="188">
         <f>+'CONCRETO EN CUNETAS'!E70</f>
@@ -4190,7 +4291,7 @@
       </c>
       <c r="C20" s="184" t="n"/>
       <c r="D20" s="190" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E20" s="188">
         <f>+'CONCRETO EN CUNETAS'!M22</f>
@@ -4228,7 +4329,7 @@
       </c>
       <c r="C21" s="184" t="n"/>
       <c r="D21" s="190" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E21" s="188">
         <f>+'CONCRETO EN CUNETAS'!M34</f>
@@ -4923,6 +5024,326 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27" customHeight="1">
+      <c r="A1" s="359" t="inlineStr">
+        <is>
+          <t>CUNETAS - ACORTAMIENTO EN LA LLEGADA AL COLECTOR PLUVIAL FRONTAL</t>
+        </is>
+      </c>
+      <c r="B1" s="360" t="n"/>
+      <c r="C1" s="360" t="n"/>
+      <c r="D1" s="360" t="n"/>
+      <c r="E1" s="360" t="n"/>
+      <c r="F1" s="360" t="n"/>
+      <c r="G1" s="360" t="n"/>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="361" t="inlineStr">
+        <is>
+          <t>ENTIDAD</t>
+        </is>
+      </c>
+      <c r="B2" s="362" t="n"/>
+      <c r="C2" s="363">
+        <f>+RESUMEN!B4</f>
+        <v/>
+      </c>
+      <c r="D2" s="362" t="n"/>
+      <c r="E2" s="362" t="n"/>
+      <c r="F2" s="362" t="n"/>
+      <c r="G2" s="362" t="n"/>
+    </row>
+    <row r="3" ht="59" customHeight="1">
+      <c r="A3" s="361" t="inlineStr">
+        <is>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="B3" s="362" t="n"/>
+      <c r="C3" s="363">
+        <f>+RESUMEN!B5</f>
+        <v/>
+      </c>
+      <c r="D3" s="362" t="n"/>
+      <c r="E3" s="362" t="n"/>
+      <c r="F3" s="362" t="n"/>
+      <c r="G3" s="362" t="n"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="361" t="inlineStr">
+        <is>
+          <t>UBICACIÓN</t>
+        </is>
+      </c>
+      <c r="B4" s="362" t="n"/>
+      <c r="C4" s="363">
+        <f>+RESUMEN!B6</f>
+        <v/>
+      </c>
+      <c r="D4" s="362" t="n"/>
+      <c r="E4" s="362" t="n"/>
+      <c r="F4" s="362" t="n"/>
+      <c r="G4" s="362" t="n"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="361" t="inlineStr">
+        <is>
+          <t>FECHA</t>
+        </is>
+      </c>
+      <c r="B5" s="362" t="n"/>
+      <c r="C5" s="364">
+        <f>+RESUMEN!B7</f>
+        <v/>
+      </c>
+      <c r="D5" s="362" t="n"/>
+      <c r="E5" s="362" t="n"/>
+      <c r="F5" s="362" t="n"/>
+      <c r="G5" s="362" t="n"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="365" t="inlineStr">
+        <is>
+          <t>Las cunetas estan dibujadas hasta la franja exterior del frente. El colector pluvial frontal ocupa esa franja, por lo que cada cuneta termina en la cara del muro lado predio del colector (ventana de empalme, lamina DP-06C) o en el muro norte de la caja de llegada CL del Hogar de Refugio (Eje 01, lamina DP-07). El tramo que caia dentro del colector se descuenta de la longitud de la cuneta en todas las hojas de este metrado (concreto, encofrado, acero, curado, rejillas, juntas, movimiento de tierras).</t>
+        </is>
+      </c>
+      <c r="B7" s="362" t="n"/>
+      <c r="C7" s="362" t="n"/>
+      <c r="D7" s="362" t="n"/>
+      <c r="E7" s="362" t="n"/>
+      <c r="F7" s="362" t="n"/>
+      <c r="G7" s="362" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="366" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B9" s="366" t="inlineStr">
+        <is>
+          <t>CUNETA</t>
+        </is>
+      </c>
+      <c r="C9" s="366" t="inlineStr">
+        <is>
+          <t>LONGITUD DIBUJADA (m)</t>
+        </is>
+      </c>
+      <c r="D9" s="366" t="inlineStr">
+        <is>
+          <t>ACORTAMIENTO (m)</t>
+        </is>
+      </c>
+      <c r="E9" s="366" t="inlineStr">
+        <is>
+          <t>LONGITUD METRADA (m)</t>
+        </is>
+      </c>
+      <c r="F9" s="366" t="inlineStr">
+        <is>
+          <t>TERMINA EN</t>
+        </is>
+      </c>
+      <c r="G9" s="366" t="inlineStr">
+        <is>
+          <t>SUSTENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="367" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="367" t="inlineStr">
+        <is>
+          <t>EJE 01</t>
+        </is>
+      </c>
+      <c r="C10" s="368" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="D10" s="368" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="E10" s="369">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="367" t="inlineStr">
+        <is>
+          <t>muro norte de la caja CL</t>
+        </is>
+      </c>
+      <c r="G10" s="370" t="inlineStr">
+        <is>
+          <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="367" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="367" t="inlineStr">
+        <is>
+          <t>EJE 04</t>
+        </is>
+      </c>
+      <c r="C11" s="368" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="D11" s="368" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="E11" s="369">
+        <f>C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="367" t="inlineStr">
+        <is>
+          <t>muro del colector (ventana)</t>
+        </is>
+      </c>
+      <c r="G11" s="370" t="inlineStr">
+        <is>
+          <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="367" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="367" t="inlineStr">
+        <is>
+          <t>EJE 06</t>
+        </is>
+      </c>
+      <c r="C12" s="368" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="D12" s="368" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E12" s="369">
+        <f>C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="367" t="inlineStr">
+        <is>
+          <t>muro del colector (ventana)</t>
+        </is>
+      </c>
+      <c r="G12" s="370" t="inlineStr">
+        <is>
+          <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="367" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="367" t="inlineStr">
+        <is>
+          <t>EJE 08</t>
+        </is>
+      </c>
+      <c r="C13" s="368" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="D13" s="368" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E13" s="369">
+        <f>C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="367" t="inlineStr">
+        <is>
+          <t>muro del colector (ventana)</t>
+        </is>
+      </c>
+      <c r="G13" s="370" t="inlineStr">
+        <is>
+          <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="367" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="367" t="inlineStr">
+        <is>
+          <t>EJE 09</t>
+        </is>
+      </c>
+      <c r="C14" s="368" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="D14" s="368" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E14" s="369">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="367" t="inlineStr">
+        <is>
+          <t>muro del colector (ventana)</t>
+        </is>
+      </c>
+      <c r="G14" s="370" t="inlineStr">
+        <is>
+          <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="371" t="inlineStr">
+        <is>
+          <t>Nota: el acortamiento se aplica al ultimo tramo de cada eje (el que llega al frente); las alturas H se mantienen las del perfil. Las cunetas de los Ejes 02, 03, 05 y 07 no llegan al frente y no cambian.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:G3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.453125" defaultRowHeight="14"/>
   <cols>
@@ -4974,7 +5395,7 @@
           <t>Cantidad de tapas</t>
         </is>
       </c>
-      <c r="B4" s="359" t="n">
+      <c r="B4" s="372" t="n">
         <v>8</v>
       </c>
       <c r="C4" s="118" t="inlineStr">
@@ -4994,7 +5415,7 @@
           <t>Largo de tapa</t>
         </is>
       </c>
-      <c r="B5" s="359" t="n">
+      <c r="B5" s="372" t="n">
         <v>0.6</v>
       </c>
       <c r="C5" s="118" t="inlineStr">
@@ -5014,7 +5435,7 @@
           <t>Ancho de tapa</t>
         </is>
       </c>
-      <c r="B6" s="359" t="n">
+      <c r="B6" s="372" t="n">
         <v>0.6</v>
       </c>
       <c r="C6" s="118" t="inlineStr">
@@ -5034,7 +5455,7 @@
           <t>Espesor de tapa</t>
         </is>
       </c>
-      <c r="B7" s="359" t="n">
+      <c r="B7" s="372" t="n">
         <v>0.1</v>
       </c>
       <c r="C7" s="118" t="inlineStr">
@@ -5054,7 +5475,7 @@
           <t>Recubrimiento considerado</t>
         </is>
       </c>
-      <c r="B8" s="359" t="n">
+      <c r="B8" s="372" t="n">
         <v>0.025</v>
       </c>
       <c r="C8" s="118" t="inlineStr">
@@ -5074,7 +5495,7 @@
           <t>Separación de varillas 3/8</t>
         </is>
       </c>
-      <c r="B9" s="359" t="n">
+      <c r="B9" s="372" t="n">
         <v>0.15</v>
       </c>
       <c r="C9" s="118" t="inlineStr">
@@ -5094,7 +5515,7 @@
           <t>Peso varilla 3/8</t>
         </is>
       </c>
-      <c r="B10" s="359" t="n">
+      <c r="B10" s="372" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="C10" s="118" t="inlineStr">
@@ -5114,7 +5535,7 @@
           <t>Longitud varilla comercial</t>
         </is>
       </c>
-      <c r="B11" s="359" t="n">
+      <c r="B11" s="372" t="n">
         <v>9</v>
       </c>
       <c r="C11" s="118" t="inlineStr">
@@ -5163,7 +5584,7 @@
           <t>Espesor de solado sumado a excavación y relleno</t>
         </is>
       </c>
-      <c r="B15" s="359" t="n">
+      <c r="B15" s="372" t="n">
         <v>0.1</v>
       </c>
       <c r="C15" s="118" t="inlineStr">
@@ -5183,7 +5604,7 @@
           <t>Factor de esponjamiento</t>
         </is>
       </c>
-      <c r="B16" s="359" t="n">
+      <c r="B16" s="372" t="n">
         <v>1.2</v>
       </c>
       <c r="C16" s="118" t="inlineStr">
@@ -5206,7 +5627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5258,7 +5679,7 @@
           <t>6 mm</t>
         </is>
       </c>
-      <c r="B4" s="360" t="n">
+      <c r="B4" s="373" t="n">
         <v>0.222</v>
       </c>
       <c r="D4" s="94" t="inlineStr">
@@ -5278,7 +5699,7 @@
           <t>8 mm</t>
         </is>
       </c>
-      <c r="B5" s="360" t="n">
+      <c r="B5" s="373" t="n">
         <v>0.395</v>
       </c>
       <c r="D5" s="94" t="inlineStr">
@@ -5298,7 +5719,7 @@
           <t>3/8"</t>
         </is>
       </c>
-      <c r="B6" s="360" t="n">
+      <c r="B6" s="373" t="n">
         <v>0.5600000000000001</v>
       </c>
     </row>
@@ -5308,7 +5729,7 @@
           <t>12 mm</t>
         </is>
       </c>
-      <c r="B7" s="360" t="n">
+      <c r="B7" s="373" t="n">
         <v>0.888</v>
       </c>
     </row>
@@ -5318,7 +5739,7 @@
           <t>1/2"</t>
         </is>
       </c>
-      <c r="B8" s="360" t="n">
+      <c r="B8" s="373" t="n">
         <v>0.994</v>
       </c>
     </row>
@@ -5328,7 +5749,7 @@
           <t>5/8"</t>
         </is>
       </c>
-      <c r="B9" s="360" t="n">
+      <c r="B9" s="373" t="n">
         <v>1.552</v>
       </c>
     </row>
@@ -5338,7 +5759,7 @@
           <t>3/4"</t>
         </is>
       </c>
-      <c r="B10" s="360" t="n">
+      <c r="B10" s="373" t="n">
         <v>2.235</v>
       </c>
     </row>
@@ -5348,7 +5769,7 @@
           <t>1"</t>
         </is>
       </c>
-      <c r="B11" s="360" t="n">
+      <c r="B11" s="373" t="n">
         <v>3.973</v>
       </c>
     </row>
@@ -5668,7 +6089,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E12" s="31" t="n">
         <v>1.4</v>
@@ -5749,7 +6170,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E15" s="31" t="n">
         <v>1.4</v>
@@ -5803,7 +6224,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E17" s="31" t="n">
         <v>1.4</v>
@@ -5857,7 +6278,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E19" s="31" t="n">
         <v>1.4</v>
@@ -5884,7 +6305,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E20" s="31" t="n">
         <v>1.4</v>
@@ -5997,7 +6418,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E25" s="31" t="n">
         <v>1.4</v>
@@ -6078,7 +6499,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E28" s="31" t="n">
         <v>1.4</v>
@@ -6132,7 +6553,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E30" s="31" t="n">
         <v>1.4</v>
@@ -6186,7 +6607,7 @@
         <v>1</v>
       </c>
       <c r="D32" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E32" s="31" t="n">
         <v>1.4</v>
@@ -6213,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E33" s="31" t="n">
         <v>1.4</v>
@@ -6348,7 +6769,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E39" s="31" t="n">
         <v>1.4</v>
@@ -6435,13 +6856,13 @@
         <v>1</v>
       </c>
       <c r="D42" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E42" s="31" t="n">
         <v>1.4</v>
       </c>
       <c r="F42" s="31" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="G42" s="31" t="n"/>
       <c r="H42" s="31" t="n"/>
@@ -6493,7 +6914,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E44" s="31" t="n">
         <v>1.4</v>
@@ -6551,7 +6972,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E46" s="31" t="n">
         <v>1.4</v>
@@ -6580,7 +7001,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E47" s="31" t="n">
         <v>1.4</v>
@@ -6767,7 +7188,7 @@
         <v>1</v>
       </c>
       <c r="D55" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E55" s="31" t="n">
         <v>0.6</v>
@@ -6848,7 +7269,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E58" s="31" t="n">
         <v>0.6</v>
@@ -6902,7 +7323,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E60" s="31" t="n">
         <v>0.6</v>
@@ -6956,7 +7377,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E62" s="31" t="n">
         <v>0.6</v>
@@ -6983,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E63" s="31" t="n">
         <v>0.6</v>
@@ -7096,7 +7517,7 @@
         <v>1</v>
       </c>
       <c r="D68" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E68" s="31" t="n">
         <v>0.8</v>
@@ -7183,13 +7604,13 @@
         <v>1</v>
       </c>
       <c r="D71" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E71" s="31" t="n">
         <v>0.8</v>
       </c>
       <c r="F71" s="31" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="G71" s="31" t="n"/>
       <c r="H71" s="31" t="n"/>
@@ -7241,7 +7662,7 @@
         <v>1</v>
       </c>
       <c r="D73" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E73" s="31" t="n">
         <v>0.8</v>
@@ -7299,7 +7720,7 @@
         <v>1</v>
       </c>
       <c r="D75" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E75" s="31" t="n">
         <v>0.8</v>
@@ -7328,7 +7749,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E76" s="31" t="n">
         <v>0.8</v>
@@ -7549,7 +7970,7 @@
         <v>1</v>
       </c>
       <c r="D85" s="31" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="E85" s="31" t="n">
         <v>0.6</v>
@@ -7630,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="D88" s="31" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="E88" s="31" t="n">
         <v>0.6</v>
@@ -7684,7 +8105,7 @@
         <v>1</v>
       </c>
       <c r="D90" s="31" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="E90" s="31" t="n">
         <v>0.6</v>
@@ -7738,7 +8159,7 @@
         <v>1</v>
       </c>
       <c r="D92" s="31" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="E92" s="31" t="n">
         <v>0.6</v>
@@ -7765,7 +8186,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="31" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="E93" s="31" t="n">
         <v>0.6</v>
@@ -9616,7 +10037,7 @@
         </is>
       </c>
       <c r="E10" s="80" t="n">
-        <v>63.31</v>
+        <v>61.2</v>
       </c>
       <c r="F10" s="319">
         <f>E10*E11*E12</f>
@@ -9758,7 +10179,7 @@
         </is>
       </c>
       <c r="E14" s="14" t="n">
-        <v>114.3</v>
+        <v>111.53</v>
       </c>
       <c r="F14" s="325" t="n"/>
       <c r="G14" s="326" t="n"/>
@@ -9816,7 +10237,7 @@
         </is>
       </c>
       <c r="E16" s="80" t="n">
-        <v>43</v>
+        <v>40.23</v>
       </c>
       <c r="F16" s="319">
         <f>E16*E17*E18</f>
@@ -9995,7 +10416,7 @@
         </is>
       </c>
       <c r="M22" s="14" t="n">
-        <v>27.4</v>
+        <v>27.34</v>
       </c>
       <c r="N22" s="322">
         <f>M22*M23*M24</f>
@@ -10119,7 +10540,7 @@
         </is>
       </c>
       <c r="M26" s="14" t="n">
-        <v>60.7</v>
+        <v>60.61</v>
       </c>
       <c r="N26" s="325" t="n"/>
       <c r="O26" s="325" t="n"/>
@@ -10182,7 +10603,7 @@
         </is>
       </c>
       <c r="M28" s="14" t="n">
-        <v>10.85</v>
+        <v>10.76</v>
       </c>
       <c r="N28" s="322">
         <f>M28*M29*M30</f>
@@ -10332,7 +10753,7 @@
         </is>
       </c>
       <c r="M34" s="80" t="n">
-        <v>17.69</v>
+        <v>17.56</v>
       </c>
       <c r="N34" s="319">
         <f>M34*M35*M36</f>
@@ -10456,7 +10877,7 @@
         </is>
       </c>
       <c r="M38" s="14" t="n">
-        <v>42.7</v>
+        <v>42.46</v>
       </c>
       <c r="N38" s="325" t="n"/>
       <c r="O38" s="326" t="n"/>
@@ -10519,7 +10940,7 @@
         </is>
       </c>
       <c r="M40" s="80" t="n">
-        <v>6.7</v>
+        <v>6.46</v>
       </c>
       <c r="N40" s="319">
         <f>M40*M41*M42</f>
@@ -10642,7 +11063,7 @@
         </is>
       </c>
       <c r="E46" s="80" t="n">
-        <v>56.69</v>
+        <v>54.48</v>
       </c>
       <c r="F46" s="319">
         <f>E46*E47*E48</f>
@@ -10776,7 +11197,7 @@
         </is>
       </c>
       <c r="E50" s="14" t="n">
-        <v>105.7</v>
+        <v>102.58</v>
       </c>
       <c r="F50" s="325" t="n"/>
       <c r="G50" s="326" t="n"/>
@@ -10832,7 +11253,7 @@
         </is>
       </c>
       <c r="E52" s="172" t="n">
-        <v>34.05</v>
+        <v>30.93</v>
       </c>
       <c r="F52" s="218">
         <f>E52*E53*E54</f>
@@ -11309,7 +11730,7 @@
         </is>
       </c>
       <c r="E70" s="80" t="n">
-        <v>52.89</v>
+        <v>52.72</v>
       </c>
       <c r="F70" s="319">
         <f>E70*E71*E72</f>
@@ -11443,7 +11864,7 @@
         </is>
       </c>
       <c r="E74" s="14" t="n">
-        <v>98.95</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="F74" s="325" t="n"/>
       <c r="G74" s="326" t="n"/>
@@ -11499,7 +11920,7 @@
         </is>
       </c>
       <c r="E76" s="80" t="n">
-        <v>66.45</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="F76" s="319">
         <f>E76*E77*E78</f>
@@ -12160,7 +12581,7 @@
         </is>
       </c>
       <c r="F16" s="14" t="n">
-        <v>36.19</v>
+        <v>33.53</v>
       </c>
       <c r="G16" s="251">
         <f>F16*F17</f>
@@ -12236,7 +12657,7 @@
         </is>
       </c>
       <c r="F18" s="14" t="n">
-        <v>27.59</v>
+        <v>25.48</v>
       </c>
       <c r="G18" s="251">
         <f>(F18*F19)+F20</f>
@@ -12304,7 +12725,7 @@
         </is>
       </c>
       <c r="F20" s="14">
-        <f>43.0*0.4</f>
+        <f>40.23*0.4</f>
         <v/>
       </c>
       <c r="G20" s="315" t="n"/>
@@ -12581,7 +13002,7 @@
         </is>
       </c>
       <c r="N27" s="85" t="n">
-        <v>27.79</v>
+        <v>24.95</v>
       </c>
       <c r="O27" s="251">
         <f>N27*N28</f>
@@ -12653,7 +13074,7 @@
         </is>
       </c>
       <c r="N29" s="85" t="n">
-        <v>20.98</v>
+        <v>18.76</v>
       </c>
       <c r="O29" s="251">
         <f>N29*N30+N31</f>
@@ -12714,7 +13135,7 @@
         </is>
       </c>
       <c r="N31" s="85">
-        <f>34.05*0.4</f>
+        <f>30.93*0.4</f>
         <v/>
       </c>
       <c r="O31" s="315" t="n"/>
@@ -12982,7 +13403,7 @@
         </is>
       </c>
       <c r="N38" s="14" t="n">
-        <v>53.82</v>
+        <v>53.6</v>
       </c>
       <c r="O38" s="251">
         <f>N38*N39</f>
@@ -13054,7 +13475,7 @@
         </is>
       </c>
       <c r="N40" s="14" t="n">
-        <v>40.53</v>
+        <v>40.36</v>
       </c>
       <c r="O40" s="251">
         <f>N40*N41+N42</f>
@@ -13116,7 +13537,7 @@
         </is>
       </c>
       <c r="N42" s="14">
-        <f>66.45*0.4</f>
+        <f>66.21*0.4</f>
         <v/>
       </c>
       <c r="O42" s="315" t="n"/>
@@ -13384,7 +13805,7 @@
         </is>
       </c>
       <c r="N49" s="14" t="n">
-        <v>8.4</v>
+        <v>8.33</v>
       </c>
       <c r="O49" s="251">
         <f>N49*N50</f>
@@ -13456,7 +13877,7 @@
         </is>
       </c>
       <c r="N51" s="14" t="n">
-        <v>6.23</v>
+        <v>6.17</v>
       </c>
       <c r="O51" s="251">
         <f>N51*N52+N53</f>
@@ -13517,7 +13938,7 @@
         </is>
       </c>
       <c r="N53" s="14">
-        <f>10.85*0.4</f>
+        <f>10.76*0.4</f>
         <v/>
       </c>
       <c r="O53" s="315" t="n"/>
@@ -13759,7 +14180,7 @@
         </is>
       </c>
       <c r="F61" s="14" t="n">
-        <v>4.94</v>
+        <v>4.76</v>
       </c>
       <c r="G61" s="251">
         <f>F61*F62</f>
@@ -13833,7 +14254,7 @@
         </is>
       </c>
       <c r="F63" s="14" t="n">
-        <v>3.6</v>
+        <v>3.47</v>
       </c>
       <c r="G63" s="251">
         <f>F63*F64+F65</f>
@@ -13899,7 +14320,7 @@
         </is>
       </c>
       <c r="F65" s="14">
-        <f>6.7*0.4</f>
+        <f>6.46*0.4</f>
         <v/>
       </c>
       <c r="G65" s="315" t="n"/>
@@ -17740,7 +18161,7 @@
         </is>
       </c>
       <c r="G13" s="107" t="n">
-        <v>37</v>
+        <v>34.23</v>
       </c>
       <c r="H13" s="106" t="inlineStr">
         <is>
@@ -17779,7 +18200,7 @@
         <v>2.06</v>
       </c>
       <c r="R13" s="107" t="n">
-        <v>2.24</v>
+        <v>2.2</v>
       </c>
       <c r="S13" s="141">
         <f>IF(B13="","",(Q13+R13)/2)</f>
@@ -18349,7 +18770,7 @@
         </is>
       </c>
       <c r="G18" s="107" t="n">
-        <v>28.55</v>
+        <v>25.43</v>
       </c>
       <c r="H18" s="106" t="inlineStr">
         <is>
@@ -18367,7 +18788,7 @@
         <v>8</v>
       </c>
       <c r="L18" s="107" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M18" s="141">
         <f>IF(B18="","",(K18+L18)/2)</f>
@@ -18388,7 +18809,7 @@
         <v>2.06</v>
       </c>
       <c r="R18" s="107" t="n">
-        <v>2.14</v>
+        <v>2.1</v>
       </c>
       <c r="S18" s="141">
         <f>IF(B18="","",(Q18+R18)/2)</f>
@@ -18841,7 +19262,7 @@
         </is>
       </c>
       <c r="G22" s="107" t="n">
-        <v>66.45</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="H22" s="106" t="inlineStr">
         <is>
@@ -19204,7 +19625,7 @@
         </is>
       </c>
       <c r="G25" s="107" t="n">
-        <v>10.85</v>
+        <v>10.76</v>
       </c>
       <c r="H25" s="106" t="inlineStr">
         <is>
@@ -19450,7 +19871,7 @@
         </is>
       </c>
       <c r="G27" s="107" t="n">
-        <v>6.7</v>
+        <v>6.46</v>
       </c>
       <c r="H27" s="106" t="inlineStr">
         <is>
@@ -20824,7 +21245,7 @@
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>37</v>
+        <v>34.23</v>
       </c>
       <c r="F10" s="202" t="n">
         <v>0.4</v>
@@ -20833,7 +21254,7 @@
         <v>0.68</v>
       </c>
       <c r="H10" s="136" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="I10" s="108">
         <f>IF(B10="","",(G10+H10)/2)</f>
@@ -21190,7 +21611,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>28.55</v>
+        <v>25.43</v>
       </c>
       <c r="F16" s="202" t="n">
         <v>0.4</v>
@@ -21199,7 +21620,7 @@
         <v>0.68</v>
       </c>
       <c r="H16" s="136" t="n">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="I16" s="108">
         <f>IF(B16="","",(G16+H16)/2)</f>
@@ -21434,7 +21855,7 @@
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.45</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="F20" s="202" t="n">
         <v>0.4</v>
@@ -21617,7 +22038,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.85</v>
+        <v>10.76</v>
       </c>
       <c r="F23" s="202" t="n">
         <v>0.4</v>
@@ -21739,7 +22160,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.7</v>
+        <v>6.46</v>
       </c>
       <c r="F25" s="202" t="n">
         <v>0.4</v>
@@ -22510,7 +22931,7 @@
         </is>
       </c>
       <c r="E10" s="136" t="n">
-        <v>37</v>
+        <v>34.23</v>
       </c>
       <c r="F10" s="176" t="n">
         <v>0</v>
@@ -22720,7 +23141,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>28.55</v>
+        <v>25.43</v>
       </c>
       <c r="F16" s="176" t="n">
         <v>0</v>
@@ -22860,7 +23281,7 @@
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.45</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="F20" s="176" t="n">
         <v>0</v>
@@ -22965,7 +23386,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.85</v>
+        <v>10.76</v>
       </c>
       <c r="F23" s="176" t="n">
         <v>0</v>
@@ -23035,7 +23456,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.7</v>
+        <v>6.46</v>
       </c>
       <c r="F25" s="176" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
CAR Varones: sin cerco perimetrico en el frente; registros exactamente en el cruce de cada cuneta (cunetas verticales); textos y juntas actualizados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C16" s="184" t="n"/>
       <c r="D16" s="190" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E16" s="188">
         <f>+'CONCRETO EN CUNETAS'!E46</f>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C18" s="184" t="n"/>
       <c r="D18" s="190" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E18" s="188">
         <f>+'CONCRETO EN CUNETAS'!E70</f>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="C20" s="184" t="n"/>
       <c r="D20" s="190" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E20" s="188">
         <f>+'CONCRETO EN CUNETAS'!M22</f>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="C21" s="184" t="n"/>
       <c r="D21" s="190" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E21" s="188">
         <f>+'CONCRETO EN CUNETAS'!M34</f>
@@ -5206,7 +5206,7 @@
         <v>105.7</v>
       </c>
       <c r="D11" s="368" t="n">
-        <v>3.12</v>
+        <v>3.39</v>
       </c>
       <c r="E11" s="369">
         <f>C11-D11</f>
@@ -5236,7 +5236,7 @@
         <v>98.95</v>
       </c>
       <c r="D12" s="368" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="E12" s="369">
         <f>C12-D12</f>
@@ -5266,7 +5266,7 @@
         <v>60.7</v>
       </c>
       <c r="D13" s="368" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E13" s="369">
         <f>C13-D13</f>
@@ -5296,7 +5296,7 @@
         <v>42.7</v>
       </c>
       <c r="D14" s="368" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="E14" s="369">
         <f>C14-D14</f>
@@ -6170,7 +6170,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E15" s="31" t="n">
         <v>1.4</v>
@@ -6224,7 +6224,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E17" s="31" t="n">
         <v>1.4</v>
@@ -6278,7 +6278,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E19" s="31" t="n">
         <v>1.4</v>
@@ -6305,7 +6305,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E20" s="31" t="n">
         <v>1.4</v>
@@ -6499,7 +6499,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E28" s="31" t="n">
         <v>1.4</v>
@@ -6553,7 +6553,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E30" s="31" t="n">
         <v>1.4</v>
@@ -6607,7 +6607,7 @@
         <v>1</v>
       </c>
       <c r="D32" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E32" s="31" t="n">
         <v>1.4</v>
@@ -6634,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E33" s="31" t="n">
         <v>1.4</v>
@@ -6856,7 +6856,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E42" s="31" t="n">
         <v>1.4</v>
@@ -6914,7 +6914,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E44" s="31" t="n">
         <v>1.4</v>
@@ -6972,7 +6972,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E46" s="31" t="n">
         <v>1.4</v>
@@ -7001,7 +7001,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E47" s="31" t="n">
         <v>1.4</v>
@@ -7269,7 +7269,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E58" s="31" t="n">
         <v>0.6</v>
@@ -7323,7 +7323,7 @@
         <v>1</v>
       </c>
       <c r="D60" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E60" s="31" t="n">
         <v>0.6</v>
@@ -7377,7 +7377,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E62" s="31" t="n">
         <v>0.6</v>
@@ -7404,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E63" s="31" t="n">
         <v>0.6</v>
@@ -7604,7 +7604,7 @@
         <v>1</v>
       </c>
       <c r="D71" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E71" s="31" t="n">
         <v>0.8</v>
@@ -7662,7 +7662,7 @@
         <v>1</v>
       </c>
       <c r="D73" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E73" s="31" t="n">
         <v>0.8</v>
@@ -7720,7 +7720,7 @@
         <v>1</v>
       </c>
       <c r="D75" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E75" s="31" t="n">
         <v>0.8</v>
@@ -7749,7 +7749,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E76" s="31" t="n">
         <v>0.8</v>
@@ -8051,7 +8051,7 @@
         <v>1</v>
       </c>
       <c r="D88" s="31" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="E88" s="31" t="n">
         <v>0.6</v>
@@ -8105,7 +8105,7 @@
         <v>1</v>
       </c>
       <c r="D90" s="31" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="E90" s="31" t="n">
         <v>0.6</v>
@@ -8159,7 +8159,7 @@
         <v>1</v>
       </c>
       <c r="D92" s="31" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="E92" s="31" t="n">
         <v>0.6</v>
@@ -8186,7 +8186,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="31" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="E93" s="31" t="n">
         <v>0.6</v>
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="M26" s="14" t="n">
-        <v>60.61</v>
+        <v>60.6</v>
       </c>
       <c r="N26" s="325" t="n"/>
       <c r="O26" s="325" t="n"/>
@@ -10603,7 +10603,7 @@
         </is>
       </c>
       <c r="M28" s="14" t="n">
-        <v>10.76</v>
+        <v>10.75</v>
       </c>
       <c r="N28" s="322">
         <f>M28*M29*M30</f>
@@ -10753,7 +10753,7 @@
         </is>
       </c>
       <c r="M34" s="80" t="n">
-        <v>17.56</v>
+        <v>17.55</v>
       </c>
       <c r="N34" s="319">
         <f>M34*M35*M36</f>
@@ -10877,7 +10877,7 @@
         </is>
       </c>
       <c r="M38" s="14" t="n">
-        <v>42.46</v>
+        <v>42.45</v>
       </c>
       <c r="N38" s="325" t="n"/>
       <c r="O38" s="326" t="n"/>
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="M40" s="80" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="N40" s="319">
         <f>M40*M41*M42</f>
@@ -11063,7 +11063,7 @@
         </is>
       </c>
       <c r="E46" s="80" t="n">
-        <v>54.48</v>
+        <v>54.29</v>
       </c>
       <c r="F46" s="319">
         <f>E46*E47*E48</f>
@@ -11197,7 +11197,7 @@
         </is>
       </c>
       <c r="E50" s="14" t="n">
-        <v>102.58</v>
+        <v>102.31</v>
       </c>
       <c r="F50" s="325" t="n"/>
       <c r="G50" s="326" t="n"/>
@@ -11253,7 +11253,7 @@
         </is>
       </c>
       <c r="E52" s="172" t="n">
-        <v>30.93</v>
+        <v>30.66</v>
       </c>
       <c r="F52" s="218">
         <f>E52*E53*E54</f>
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="E70" s="80" t="n">
-        <v>52.72</v>
+        <v>52.71</v>
       </c>
       <c r="F70" s="319">
         <f>E70*E71*E72</f>
@@ -11864,7 +11864,7 @@
         </is>
       </c>
       <c r="E74" s="14" t="n">
-        <v>98.70999999999999</v>
+        <v>98.69</v>
       </c>
       <c r="F74" s="325" t="n"/>
       <c r="G74" s="326" t="n"/>
@@ -11920,7 +11920,7 @@
         </is>
       </c>
       <c r="E76" s="80" t="n">
-        <v>66.20999999999999</v>
+        <v>66.19</v>
       </c>
       <c r="F76" s="319">
         <f>E76*E77*E78</f>
@@ -13002,7 +13002,7 @@
         </is>
       </c>
       <c r="N27" s="85" t="n">
-        <v>24.95</v>
+        <v>24.7</v>
       </c>
       <c r="O27" s="251">
         <f>N27*N28</f>
@@ -13074,7 +13074,7 @@
         </is>
       </c>
       <c r="N29" s="85" t="n">
-        <v>18.76</v>
+        <v>18.57</v>
       </c>
       <c r="O29" s="251">
         <f>N29*N30+N31</f>
@@ -13135,7 +13135,7 @@
         </is>
       </c>
       <c r="N31" s="85">
-        <f>30.93*0.4</f>
+        <f>30.66*0.4</f>
         <v/>
       </c>
       <c r="O31" s="315" t="n"/>
@@ -13403,7 +13403,7 @@
         </is>
       </c>
       <c r="N38" s="14" t="n">
-        <v>53.6</v>
+        <v>53.59</v>
       </c>
       <c r="O38" s="251">
         <f>N38*N39</f>
@@ -13475,7 +13475,7 @@
         </is>
       </c>
       <c r="N40" s="14" t="n">
-        <v>40.36</v>
+        <v>40.35</v>
       </c>
       <c r="O40" s="251">
         <f>N40*N41+N42</f>
@@ -13537,7 +13537,7 @@
         </is>
       </c>
       <c r="N42" s="14">
-        <f>66.21*0.4</f>
+        <f>66.19*0.4</f>
         <v/>
       </c>
       <c r="O42" s="315" t="n"/>
@@ -13805,7 +13805,7 @@
         </is>
       </c>
       <c r="N49" s="14" t="n">
-        <v>8.33</v>
+        <v>8.32</v>
       </c>
       <c r="O49" s="251">
         <f>N49*N50</f>
@@ -13938,7 +13938,7 @@
         </is>
       </c>
       <c r="N53" s="14">
-        <f>10.76*0.4</f>
+        <f>10.75*0.4</f>
         <v/>
       </c>
       <c r="O53" s="315" t="n"/>
@@ -14180,7 +14180,7 @@
         </is>
       </c>
       <c r="F61" s="14" t="n">
-        <v>4.76</v>
+        <v>4.75</v>
       </c>
       <c r="G61" s="251">
         <f>F61*F62</f>
@@ -14254,7 +14254,7 @@
         </is>
       </c>
       <c r="F63" s="14" t="n">
-        <v>3.47</v>
+        <v>3.46</v>
       </c>
       <c r="G63" s="251">
         <f>F63*F64+F65</f>
@@ -14320,7 +14320,7 @@
         </is>
       </c>
       <c r="F65" s="14">
-        <f>6.46*0.4</f>
+        <f>6.45*0.4</f>
         <v/>
       </c>
       <c r="G65" s="315" t="n"/>
@@ -18770,7 +18770,7 @@
         </is>
       </c>
       <c r="G18" s="107" t="n">
-        <v>25.43</v>
+        <v>25.16</v>
       </c>
       <c r="H18" s="106" t="inlineStr">
         <is>
@@ -19262,7 +19262,7 @@
         </is>
       </c>
       <c r="G22" s="107" t="n">
-        <v>66.20999999999999</v>
+        <v>66.19</v>
       </c>
       <c r="H22" s="106" t="inlineStr">
         <is>
@@ -19625,7 +19625,7 @@
         </is>
       </c>
       <c r="G25" s="107" t="n">
-        <v>10.76</v>
+        <v>10.75</v>
       </c>
       <c r="H25" s="106" t="inlineStr">
         <is>
@@ -19871,7 +19871,7 @@
         </is>
       </c>
       <c r="G27" s="107" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="H27" s="106" t="inlineStr">
         <is>
@@ -21611,7 +21611,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>25.43</v>
+        <v>25.16</v>
       </c>
       <c r="F16" s="202" t="n">
         <v>0.4</v>
@@ -21855,7 +21855,7 @@
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.20999999999999</v>
+        <v>66.19</v>
       </c>
       <c r="F20" s="202" t="n">
         <v>0.4</v>
@@ -22038,7 +22038,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.76</v>
+        <v>10.75</v>
       </c>
       <c r="F23" s="202" t="n">
         <v>0.4</v>
@@ -22160,7 +22160,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="F25" s="202" t="n">
         <v>0.4</v>
@@ -23141,7 +23141,7 @@
         </is>
       </c>
       <c r="E16" s="136" t="n">
-        <v>25.43</v>
+        <v>25.16</v>
       </c>
       <c r="F16" s="176" t="n">
         <v>0</v>
@@ -23281,7 +23281,7 @@
         </is>
       </c>
       <c r="E20" s="136" t="n">
-        <v>66.20999999999999</v>
+        <v>66.19</v>
       </c>
       <c r="F20" s="176" t="n">
         <v>0</v>
@@ -23386,7 +23386,7 @@
         </is>
       </c>
       <c r="E23" s="136" t="n">
-        <v>10.76</v>
+        <v>10.75</v>
       </c>
       <c r="F23" s="176" t="n">
         <v>0</v>
@@ -23456,7 +23456,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="F25" s="176" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Varones: empalmes sobre las lineas reales de las cunetas (verticales), Eje 09 en x=349254.72; caudales en textos calculados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_CAR_VARONES_CUNETAS.xlsx
@@ -4329,7 +4329,7 @@
       </c>
       <c r="C21" s="184" t="n"/>
       <c r="D21" s="190" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E21" s="188">
         <f>+'CONCRETO EN CUNETAS'!M34</f>
@@ -5296,7 +5296,7 @@
         <v>42.7</v>
       </c>
       <c r="D14" s="368" t="n">
-        <v>0.25</v>
+        <v>0.04</v>
       </c>
       <c r="E14" s="369">
         <f>C14-D14</f>
@@ -6305,7 +6305,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E20" s="31" t="n">
         <v>1.4</v>
@@ -6634,7 +6634,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E33" s="31" t="n">
         <v>1.4</v>
@@ -7001,7 +7001,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E47" s="31" t="n">
         <v>1.4</v>
@@ -7404,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E63" s="31" t="n">
         <v>0.6</v>
@@ -7749,7 +7749,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E76" s="31" t="n">
         <v>0.8</v>
@@ -8186,7 +8186,7 @@
         <v>1</v>
       </c>
       <c r="D93" s="31" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="E93" s="31" t="n">
         <v>0.6</v>
@@ -10753,7 +10753,7 @@
         </is>
       </c>
       <c r="M34" s="80" t="n">
-        <v>17.55</v>
+        <v>17.67</v>
       </c>
       <c r="N34" s="319">
         <f>M34*M35*M36</f>
@@ -10877,7 +10877,7 @@
         </is>
       </c>
       <c r="M38" s="14" t="n">
-        <v>42.45</v>
+        <v>42.66</v>
       </c>
       <c r="N38" s="325" t="n"/>
       <c r="O38" s="326" t="n"/>
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="M40" s="80" t="n">
-        <v>6.45</v>
+        <v>6.66</v>
       </c>
       <c r="N40" s="319">
         <f>M40*M41*M42</f>
@@ -14180,7 +14180,7 @@
         </is>
       </c>
       <c r="F61" s="14" t="n">
-        <v>4.75</v>
+        <v>4.91</v>
       </c>
       <c r="G61" s="251">
         <f>F61*F62</f>
@@ -14254,7 +14254,7 @@
         </is>
       </c>
       <c r="F63" s="14" t="n">
-        <v>3.46</v>
+        <v>3.58</v>
       </c>
       <c r="G63" s="251">
         <f>F63*F64+F65</f>
@@ -14320,7 +14320,7 @@
         </is>
       </c>
       <c r="F65" s="14">
-        <f>6.45*0.4</f>
+        <f>6.66*0.4</f>
         <v/>
       </c>
       <c r="G65" s="315" t="n"/>
@@ -19871,7 +19871,7 @@
         </is>
       </c>
       <c r="G27" s="107" t="n">
-        <v>6.45</v>
+        <v>6.66</v>
       </c>
       <c r="H27" s="106" t="inlineStr">
         <is>
@@ -22160,7 +22160,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.45</v>
+        <v>6.66</v>
       </c>
       <c r="F25" s="202" t="n">
         <v>0.4</v>
@@ -23456,7 +23456,7 @@
         </is>
       </c>
       <c r="E25" s="136" t="n">
-        <v>6.45</v>
+        <v>6.66</v>
       </c>
       <c r="F25" s="176" t="n">
         <v>0</v>

</xml_diff>